<commit_message>
reconcile supplementary classifications and risk tests
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S2_Guideline_Concordance.xlsx
+++ b/Supplementary_Data_S2_Guideline_Concordance.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25600" windowHeight="10480" tabRatio="600" firstSheet="4" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Questions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2_LLM_responses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_GC_scores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_Model_summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_Question_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Reliability" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_Reference_standards" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_Sources" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S9_Rubric" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S10_Question_specific_criteria" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="S1_Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="S2_LLM_responses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="S3_GC_scores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="S4_Model_summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="S5_Question_summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="S6_Reliability" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="S7_Reference_standards" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="S8_Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="S9_Rubric" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="S10_Question_specific_criteria" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S1_Questions'!$A$1:$D$21</definedName>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -4913,7 +4913,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -5393,7 +5393,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -6225,7 +6225,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -6831,7 +6831,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -7695,7 +7695,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>症状识别与就医警示</t>
+          <t>Symptom recognition and warning signs</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -8175,7 +8175,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -9039,7 +9039,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -9135,7 +9135,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>预后、复发与疾病进展</t>
+          <t>Prognosis and recurrence</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -9231,7 +9231,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -9999,7 +9999,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -10287,7 +10287,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -10671,7 +10671,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>治疗决策与治疗相关问题</t>
+          <t>Treatment decision-related information</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -11343,7 +11343,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Nursing education/supportive care</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -11823,7 +11823,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -12015,7 +12015,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -12303,7 +12303,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>术后康复与支持照护</t>
+          <t>Postoperative recovery and home care</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">

</xml_diff>

<commit_message>
finish supplementary metadata and classification audit
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S2_Guideline_Concordance.xlsx
+++ b/Supplementary_Data_S2_Guideline_Concordance.xlsx
@@ -14209,7 +14209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -14239,6 +14239,16 @@
           <t>URL</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Version or publication/update date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Available before 2026-03-10 cutoff</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -14261,6 +14271,16 @@
           <t>https://uroweb.org/guidelines/non-muscle-invasive-bladder-cancer</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025 edition; official archive</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -14283,6 +14303,16 @@
           <t>https://uroweb.org/guidelines/muscle-invasive-and-metastatic-bladder-cancer</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025 edition; official archive</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -14305,6 +14335,16 @@
           <t>https://www.auanet.org/guidelines-and-quality/guidelines/bladder-cancer-non-muscle-invasive-guideline</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2024 Amendment; final PDF dated 2024-09-24</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -14327,6 +14367,16 @@
           <t>https://www.cancer.gov/types/bladder/hp/bladder-treatment-pdq</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Updated 2025-05-02</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -14349,6 +14399,16 @@
           <t>https://www.fda.gov/drugs/resources-information-approved-drugs/fda-approves-erdafitinib-locally-advanced-or-metastatic-urothelial-carcinoma</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Published 2024-01-19</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -14371,6 +14431,16 @@
           <t>https://www.mskcc.org/cancer-care/patient-education/about-your-urostomy</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Last updated 2025-01-28</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -14393,6 +14463,16 @@
           <t>https://www.mskcc.org/cancer-care/patient-education/changing-urostomy-pouching-system-at-home</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Last updated 2025-01-28</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -14413,6 +14493,48 @@
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>https://www.nhsa.gov.cn/art/2025/12/7/art_53_18971.html</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Published 2025-12-07</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NCCN Bladder Cancer guidance</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Formal clinical guideline</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bladder cancer treatment and management cross-check</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.nccn.org/guidelines/guidelines-detail?category=1&amp;id=145</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Version 3.2024</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clean public supplementary materials and align question numbering
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S2_Guideline_Concordance.xlsx
+++ b/Supplementary_Data_S2_Guideline_Concordance.xlsx
@@ -20,6 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S1_Questions'!$A$1:$D$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'S2_LLM_responses'!$A$1:$G$61</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'S2_LLM_responses'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S3_GC_scores'!$A$1:$Z$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S4_Model_summary'!$A$1:$Q$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S5_Question_summary'!$A$1:$G$21</definedName>
@@ -682,7 +683,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -695,6 +696,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2602,7 +2606,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
@@ -2614,6 +2618,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="100" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2681,16 +2686,15 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2.血尿就是膀胱癌吗？
-这是一个非常重要且常见的问题。直接回答您：血尿不一定是膀胱癌，但血尿，尤其是无痛性肉眼血尿，是膀胱癌最重要的警示信号，必须严肃对待，立即就医排查。
+          <t>这是一个非常重要且常见的问题。直接回答您：血尿不一定是膀胱癌，但血尿，尤其是无痛性肉眼血尿，是膀胱癌最重要的警示信号，必须严肃对待，立即就医排查。
 您可以这样理解：血尿是身体发出的“警报灯”，它告诉您泌尿系统某个地方可能出了问题，但问题的性质可能是良性的，也可能是恶性的。
-血尿可能的原因分为两大类：
-一、良性原因（更常见）
+ 血尿可能的原因分为两大类：
+ 一、良性原因（更常见）
 这些是导致血尿的绝大多数情况：
 1.  泌尿系统感染：如膀胱炎、尿道炎、肾盂肾炎。通常伴有尿频、尿急、尿痛、发热等症状。
 2.  泌尿系统结石：肾结石、输尿管结石、膀胱结石。结石移动时划伤黏膜引起出血，常伴有剧烈腰痛或腹痛。
@@ -2698,23 +2702,23 @@
 4.  肾脏疾病：如肾小球肾炎、IgA肾病等，常表现为镜下血尿（肉眼看不见，化验才发现），可能伴有蛋白尿、高血压、浮肿。
 5.  剧烈运动：有时可引起运动性血尿，通常休息后消失。
 6.  药物影响：如服用抗凝药（阿司匹林、华法林等）、某些化疗药或中药。
-二、恶性原因（必须首先排除）
+ 二、恶性原因（必须首先排除）
 1.  膀胱癌：无痛性肉眼血尿是其最典型、最早期的症状。血尿可能时有时无，间歇出现，容易让人忽视。
 2.  肾癌
 3.  输尿管癌
 4.  前列腺癌
-如何判断血尿的危险程度？——关注以下几个特征：
+ 如何判断血尿的危险程度？——关注以下几个特征：
 1.  是否伴有疼痛：
-无痛性肉眼血尿：这是最需要警惕的信号，往往是泌尿系统肿瘤（如膀胱癌）的特点。因为肿瘤出血时，早期通常不引起疼痛。
-伴有疼痛的血尿：更多指向感染或结石等良性问题。
+    无痛性肉眼血尿：这是最需要警惕的信号，往往是泌尿系统肿瘤（如膀胱癌）的特点。因为肿瘤出血时，早期通常不引起疼痛。
+       伴有疼痛的血尿：更多指向感染或结石等良性问题。
 2.  血尿的形态：
-全程血尿：排尿从开始到结束都是红色，提示出血部位可能在膀胱或以上（肾脏、输尿管）。
-初始血尿：仅排尿开始时带血，之后变清，提示问题可能在前尿道。
-终末血尿：排尿最后部分带血，提示问题可能在膀胱三角区或后尿道。
+    全程血尿：排尿从开始到结束都是红色，提示出血部位可能在膀胱或以上（肾脏、输尿管）。
+    初始血尿：仅排尿开始时带血，之后变清，提示问题可能在前尿道。
+    终末血尿：排尿最后部分带血，提示问题可能在膀胱三角区或后尿道。
 3.  血尿中是否有血块：
-如果有条状或蚯蚓状血块，可能来自肾脏或输尿管。
-如果血块较大、不规则，可能来自膀胱。
-出现血尿，您应该怎么做？（行动指南）
+    如果有条状或蚯蚓状血块，可能来自肾脏或输尿管。
+    如果血块较大、不规则，可能来自膀胱。
+ 出现血尿，您应该怎么做？（行动指南）
 第一步：立即就医，不要等待！
 不要因为血尿自行消失而掉以轻心。尤其是无痛性、间歇性的血尿，更不能拖延。
 第二步：挂对科室
@@ -2725,7 +2729,7 @@
 2.  泌尿系统超声（B超）：无创、经济，是首选的筛查手段，可以发现较大的肿瘤、结石、积水等。
 3.  CT尿路成像（CTU）：更精确的检查，可以清晰显示整个泌尿系统的形态，是诊断肿瘤和结石的“利器”。
 4.  膀胱镜检：这是诊断膀胱癌的“金标准”。医生通过一根细小的镜子经尿道进入膀胱，直接观察膀胱内部情况。如有可疑肿瘤，可以直接取活检明确病理诊断。
-总结
+ 总结
 血尿 ≠ 膀胱癌，但血尿（尤其无痛性血尿） ≈ 必须尽快看泌尿外科医生的红灯信号。
 请务必摒弃“血尿停了就没事了”的错误观念。早期膀胱癌治疗效果非常好，而延误诊断则可能导致严重后果。及时、彻底的检查，是为了排除最坏的可能性，或者在最早期发现它，从而获得最佳的治疗效果。
 一句话：看到血尿，不要猜，不要拖，马上去看医生。
@@ -2738,13 +2742,13 @@
 血液系统疾病：血小板减少、白血病、血友病
 药物影响：抗凝药物（阿司匹林、华法林）
 其他：系统性红斑狼疮、过敏性紫癜
-需要警惕的信号
+需要警惕的信号 
 出现以下情况应及时就医：
 无痛性肉眼血尿：全程血尿，不伴疼痛
 血尿反复发作：间歇性出现，自行缓解后又复发
 年龄大于40岁：中老年人血尿需警惕肿瘤
 伴有其他症状：尿频、尿急、尿痛、腰痛、消瘦
-诊断建议
+诊断建议 
 医生会通过尿常规、泌尿系B超、CT、膀胱镜等检查明确病因。特别是中老年人出现无痛性血尿，必须排除泌尿系统肿瘤的可能。早期发现、早期治疗是提高治愈率的关键。</t>
         </is>
       </c>
@@ -2782,8 +2786,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2.血尿就是膀胱癌吗
-"血尿不一定就是膀胱癌，但它是膀胱癌最常见的首发症状，同时也可能由多种其他泌尿系统或全身性疾病引起。
+          <t>血尿不一定就是膀胱癌，但它是膀胱癌最常见的首发症状，同时也可能由多种其他泌尿系统或全身性疾病引起。
 可以从血尿的表现和对应的常见病因来区分：
 膀胱癌相关的血尿特点
 膀胱癌引起的血尿多为间歇性、无痛性的肉眼血尿，尿液中可能混有血丝或血块，可能出现一次后自行消失，容易让人忽视，之后又反复出现。
@@ -2831,8 +2834,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>血尿就是膀胱癌吗？
-血尿并不一定是膀胱癌，但它是膀胱癌的重要警示信号之一。
+          <t>血尿并不一定是膀胱癌，但它是膀胱癌的重要警示信号之一。
 为什么会出现血尿？
 血尿是指尿液中红细胞数量异常增多，可能由多种原因引起，包括：
 泌尿系统疾病：如膀胱炎、尿道炎、肾结石、输尿管结石、前列腺增生、肾炎等。
@@ -2883,37 +2885,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>4.男性膀胱癌症状的早期表现
-对于男性膀胱癌，早期发现至关重要，因为早期（非肌层浸润性）膀胱癌的治疗效果非常好。其早期症状相对明确，但有一个核心特点：可能不引起疼痛，且时有时无，容易被忽视或误认为“上火”而延误就医。
+          <t>对于男性膀胱癌，早期发现至关重要，因为早期（非肌层浸润性）膀胱癌的治疗效果非常好。其早期症状相对明确，但有一个核心特点：可能不引起疼痛，且时有时无，容易被忽视或误认为“上火”而延误就医。
 以下是男性膀胱癌最常见的早期表现，请务必牢记：
 最核心、最典型的早期信号（占80%以上）
 无痛性肉眼血尿
 这是膀胱癌最首要、最关键的警报。
 “无痛”：排尿时通常没有疼痛或烧灼感。正因为不疼，很多人会掉以轻心。
 “肉眼”：眼睛可以直接看到尿液颜色异常。颜色可能呈：
-洗肉水样（淡红色）
-粉红色
-浓茶色
-甚至鲜红色，严重时可有血块。
+ 洗肉水样（淡红色）
+ 粉红色
+ 浓茶色
+ 甚至鲜红色，严重时可有血块。
 “间歇性”：这是最大的“陷阱”。血尿可能今天出现，明天或过几天就自行消失了。但这绝不代表问题解决了，肿瘤可能仍在生长。这种间歇性会给人“好了”的假象，导致延误数月甚至更久。
 其他可能出现的早期伴随症状
 这些症状可能单独出现，但更多时候是与血尿同时或交替出现：
 1.膀胱刺激症状（易被误诊为感染）
-尿频（排尿次数明显增多）
-尿急（一有尿意就憋不住）
-尿痛（排尿时有灼热或刺痛感）
-关键区别：普通的膀胱炎经抗感染治疗后，这些症状会很快消失。如果经规范消炎治疗后，症状（尤其伴有血尿时）仍持续或反复，必须警惕膀胱癌可能。
+  尿频（排尿次数明显增多）
+  尿急（一有尿意就憋不住）
+  尿痛（排尿时有灼热或刺痛感）
+  关键区别：普通的膀胱炎经抗感染治疗后，这些症状会很快消失。如果经规范消炎治疗后，症状（尤其伴有血尿时）仍持续或反复，必须警惕膀胱癌可能。
 2.排尿异常或梗阻
-排尿费力、尿线变细、排尿等待。
-感觉排尿不尽。
-这些症状在早期可能不明显，当肿瘤长在膀胱颈口或前列腺附近时较易出现。
+  排尿费力、尿线变细、排尿等待。
+  感觉排尿不尽。
+  这些症状在早期可能不明显，当肿瘤长在膀胱颈口或前列腺附近时较易出现。
 3.腰部或下背部酸胀
-如果肿瘤位于输尿管口附近，引起一侧肾脏的尿液引流不畅（肾积水），可能导致患侧腰部酸胀不适。这是一个需要警惕的信号。
+  如果肿瘤位于输尿管口附近，引起一侧肾脏的尿液引流不畅（肾积水），可能导致患侧腰部酸胀不适。这是一个需要警惕的信号。
 总结与重要提示
 1.“无痛性间歇肉眼血尿”是头号警报：只要出现过一次，无论后来是否消失，都必须去泌尿外科彻底检查。
 2.不要自我诊断：切勿自行判断为“上火”、“肾炎”或“前列腺炎”而服用药物，掩盖病情。
@@ -2956,8 +2957,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌症状的早期表现
-"男性膀胱癌的早期症状以间歇性、无痛性肉眼血尿为核心表现，部分患者可能伴随轻微的尿路刺激症状，具体如下：
+          <t>男性膀胱癌的早期症状以间歇性、无痛性肉眼血尿为核心表现，部分患者可能伴随轻微的尿路刺激症状，具体如下：
 间歇性、无痛性肉眼血尿
 这是膀胱癌最典型、最常见的早期症状，发生率高达 80% 以上。
 尿液颜色呈淡红色、洗肉水样，严重时可能混有血丝或血块，排尿时没有疼痛感，很容易被忽视。
@@ -2967,7 +2967,7 @@
 部分早期患者，尤其是肿瘤位置靠近膀胱三角区时，可能出现轻度的尿频、尿急，即排尿次数增多、有尿意时需尽快排尿，但症状通常不明显，容易与普通膀胱炎混淆。
 其他少见的早期表现
 极少数情况下，肿瘤堵塞输尿管开口，可能引起轻度的腰部酸胀、隐痛，但这种情况在早期膀胱癌中较为罕见。
-需要注意的是，男性膀胱癌的早期症状缺乏特异性，很容易与尿路结石、前列腺增生、膀胱炎等疾病的症状混淆。一旦出现上述异常，建议及时做泌尿系超声、膀胱镜等检查，明确病因，避免漏诊。"</t>
+需要注意的是，男性膀胱癌的早期症状缺乏特异性，很容易与尿路结石、前列腺增生、膀胱炎等疾病的症状混淆。一旦出现上述异常，建议及时做泌尿系超声、膀胱镜等检查，明确病因，避免漏诊。</t>
         </is>
       </c>
     </row>
@@ -3004,8 +3004,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌症状的早期表现
-无痛性肉眼血尿：这是膀胱癌最常见、也是最早出现的症状。
+          <t>无痛性肉眼血尿：这是膀胱癌最常见、也是最早出现的症状。
 特点：尿液呈洗肉水样、茶色或鲜红色，通常不伴有疼痛、尿频、尿急、尿痛等不适。
 注意：这种血尿可能是间歇性的，时有时无，容易被忽视。
 排尿习惯改变：
@@ -3051,13 +3050,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>12.膀胱癌除了血尿，还会有尿频尿急尿痛、夜尿增多这些症状吗？
-是的，完全正确。除了血尿，膀胱癌确实经常引起尿频、尿急、尿痛、夜尿增多等下尿路刺激症状。这些症状虽然在尿路感染或前列腺增生等疾病中更常见，但当肿瘤发展到一定程度时，它们也会成为膀胱癌的重要信号。下面详细解释为什么膀胱癌会引起这些症状，以及如何与其他疾病区分：为什么膀胱癌会引起这些症状？
+          <t>是的，完全正确。除了血尿，膀胱癌确实经常引起尿频、尿急、尿痛、夜尿增多等下尿路刺激症状。这些症状虽然在尿路感染或前列腺增生等疾病中更常见，但当肿瘤发展到一定程度时，它们也会成为膀胱癌的重要信号。下面详细解释为什么膀胱癌会引起这些症状，以及如何与其他疾病区分：为什么膀胱癌会引起这些症状？
 1.  肿瘤的物理刺激： 尿频、尿急：肿瘤长在膀胱壁上，就像膀胱里长了一个“异物”，会不断刺激膀胱壁的感受器，向大脑发送“需要排尿”的错误信号。夜尿增多：白天活动时，尿液对肿瘤的冲刷作用较强。夜间平躺时，肿瘤可能更容易直接接触并刺激到膀胱的敏感区域（如三角区）。
 2.  肿瘤侵犯和炎症：尿痛（排尿疼痛）：当肿瘤发生坏死、溃疡或合并感染时，排出的尿液（可能含有坏死组织、血块、细菌等）会刺激尿道，引起烧灼感或疼痛。疼痛：除了排尿痛，如果肿瘤侵犯较深，患者还可能感到下腹部或耻骨上方的持续性钝痛。
 3.  肿瘤堵塞出口：排尿困难、尿线变细、尿不尽感：当肿瘤长在膀胱颈或尿道内口附近时，会像“塞子”一样堵塞尿流通道，导致类似前列腺增生的排尿梗阻症状。
@@ -3067,14 +3065,14 @@
 症状持续且常规治疗无效：如果按照“尿路感染”进行抗生素治疗后，尿频、尿急、尿痛等症状没有明显改善或很快复发，必须警惕肿瘤的可能。
 伴有其他全身症状：晚期膀胱癌可能伴有体重不明原因下降、持续疲劳、骨盆或腰部疼痛、下肢水肿（肿瘤压迫淋巴或血管）等。
 高风险人群：长期吸烟者、有化工染料（如苯胺）接触史者、慢性膀胱炎或血吸虫病史者、有盆腔放疗史者、年龄较大（尤其50岁以上）的男性，出现上述症状时应格外重视。
-如何与常见疾病区分？
+ 如何与常见疾病区分？
 | 症状 | 膀胱癌 | 急性膀胱炎 | 前列腺增生（男性） |
 | 血尿 | 常见，无痛性、间歇性 | 可能有，但通常伴有剧烈尿痛 | 少见，若有多为终末血尿 |
 | 尿频尿急 | 常见，持续性 | 非常显著，突发 | 常见，以夜尿增多为主 |
 | 尿痛 | 可能，尤其合并感染时 | 剧烈，烧灼感 | 少见，除非合并感染 |
 | 其他特点 | 症状顽固，抗生素无效 | 起病急，抗生素有效 | 排尿费力、尿线细、尿不尽 |
 | 关键点 | 必须通过膀胱镜排除 | 尿检可见大量白细胞 | 通过B超和指诊可诊断 |
-总结与建议
+ 总结与建议
 1.  膀胱癌的症状谱很广：它不仅表现为“无痛血尿”，尿频、尿急、尿痛、夜尿增多同样是其常见症状，尤其是当肿瘤位于膀胱三角区（靠近尿道口）时。
 2.  “治疗后无效”是关键：如果下尿路症状反复发作，且常规抗炎治疗效果不佳，绝不能掉以轻心。
 3.  明确诊断是关键：尿常规、泌尿系B超是初步筛查，但诊断膀胱癌的“金标准”是膀胱镜检查 + 病理活检。如果B超发现膀胱内有占位（肿瘤），或者尿脱落细胞学检查发现癌细胞，就必须进行膀胱镜检查。
@@ -3115,8 +3113,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌除了血尿，还会有尿频尿急尿痛、夜尿增多这些症状吗？
-"是的，膀胱癌除了典型的无痛性肉眼血尿外，尿频、尿急、尿痛、夜尿增多这些下尿路刺激症状也是较为常见的表现，其出现与肿瘤的位置、大小、浸润程度及合并症密切相关。
+          <t>是的，膀胱癌除了典型的无痛性肉眼血尿外，尿频、尿急、尿痛、夜尿增多这些下尿路刺激症状也是较为常见的表现，其出现与肿瘤的位置、大小、浸润程度及合并症密切相关。
 症状出现的核心原因
 肿瘤直接刺激膀胱黏膜
 膀胱壁的黏膜富含神经末梢，当肿瘤（尤其是表浅性、多发性肿瘤或原位癌）生长时，会直接压迫、刺激黏膜，引发膀胱逼尿肌的不自主收缩，进而导致尿频、尿急。
@@ -3131,7 +3128,7 @@
 若膀胱癌患者以血尿 + 下尿路刺激症状为首发表现，往往提示肿瘤可能为原位癌或多发性浅表肿瘤，这类情况恶性程度相对较高，需尽快完善膀胱镜检查明确诊断。
 若治疗后症状再次出现，可能提示肿瘤复发或合并感染，需及时复查。
 与良性疾病的鉴别
-需要注意的是，尿频、尿急、尿痛等症状并非膀胱癌特有，也可见于良性前列腺增生、慢性膀胱炎、间质性膀胱炎等疾病，因此需结合血尿特点（膀胱癌多为无痛性、间歇性肉眼血尿）及影像学、内镜检查进一步区分"</t>
+需要注意的是，尿频、尿急、尿痛等症状并非膀胱癌特有，也可见于良性前列腺增生、慢性膀胱炎、间质性膀胱炎等疾病，因此需结合血尿特点（膀胱癌多为无痛性、间歇性肉眼血尿）及影像学、内镜检查进一步区分</t>
         </is>
       </c>
     </row>
@@ -3168,19 +3165,18 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌除了血尿，还会有尿频尿急尿痛、夜尿增多这些症状吗？
-是的，膀胱癌除了血尿之外，确实可能出现尿频、尿急、尿痛、夜尿增多等症状。
+          <t>是的，膀胱癌除了血尿之外，确实可能出现尿频、尿急、尿痛、夜尿增多等症状。
 这些症状的出现主要与肿瘤的位置、大小以及对膀胱黏膜的刺激有关：
 1.  尿频、尿急、尿痛：
-◦   当肿瘤生长在膀胱三角区、颈部或靠近尿道口时，容易刺激膀胱黏膜，引起膀胱逼尿肌不稳定收缩，从而导致尿频、尿急。
-◦   如果肿瘤合并感染或坏死，或者肿瘤表面破溃出血，也可能引起尿痛。
-◦   这些症状在膀胱癌患者中并不少见，尤其是在肿瘤较大、位置特殊或合并感染的情况下。
+    ◦   当肿瘤生长在膀胱三角区、颈部或靠近尿道口时，容易刺激膀胱黏膜，引起膀胱逼尿肌不稳定收缩，从而导致尿频、尿急。
+    ◦   如果肿瘤合并感染或坏死，或者肿瘤表面破溃出血，也可能引起尿痛。
+    ◦   这些症状在膀胱癌患者中并不少见，尤其是在肿瘤较大、位置特殊或合并感染的情况下。
 2.  夜尿增多：
-◦   夜尿增多也是膀胱癌可能出现的症状之一。这可能与肿瘤刺激膀胱，导致膀胱容量减少或膀胱逼尿肌功能异常有关。
-◦   此外，如果肿瘤导致上尿路积水，影响肾功能，也可能间接引起夜尿增多。
+    ◦   夜尿增多也是膀胱癌可能出现的症状之一。这可能与肿瘤刺激膀胱，导致膀胱容量减少或膀胱逼尿肌功能异常有关。
+    ◦   此外，如果肿瘤导致上尿路积水，影响肾功能，也可能间接引起夜尿增多。
 需要注意的是：
-•   尿频、尿急、尿痛、夜尿增多这些症状并非膀胱癌所特有，也常见于其他泌尿系统疾病，如膀胱炎、尿道炎、膀胱结石、前列腺增生等。
-•   因此，如果出现这些症状，尤其是无痛性肉眼血尿，应及时就医，进行相关检查（如尿常规、尿细胞学检查、超声、膀胱镜等），以明确病因，避免延误病情。
+尿频、尿急、尿痛、夜尿增多这些症状并非膀胱癌所特有，也常见于其他泌尿系统疾病，如膀胱炎、尿道炎、膀胱结石、前列腺增生等。
+因此，如果出现这些症状，尤其是无痛性肉眼血尿，应及时就医，进行相关检查（如尿常规、尿细胞学检查、超声、膀胱镜等），以明确病因，避免延误病情。
 总的来说，膀胱癌患者除了血尿外，确实可能出现尿频、尿急、尿痛、夜尿增多等症状，但这些症状并非特异性，需要结合其他检查和临床表现来综合判断。</t>
         </is>
       </c>
@@ -3213,43 +3209,42 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>18.膀胱癌患者尿血有血块，是不是很严重？怎么快速止血？
-看到尿血且有血块，您或您的家人一定非常紧张和担忧。这是一个需要立即严肃对待的紧急情况。
+          <t>看到尿血且有血块，您或您的家人一定非常紧张和担忧。这是一个需要立即严肃对待的紧急情况。
 请先遵循以下核心行动原则：不要自行处理，首要任务是立即就医！
 下面我将分两部分为您详细解释：为什么这很严重，以及正确的处理步骤。
-第一部分：为什么尿血有血块很严重？
+ 第一部分：为什么尿血有血块很严重？
 是的，这是一个危险的信号，通常意味着出血量较大，且可能存在急性风险。
 1.  出血量大：血液能在膀胱内凝结成块，说明出血速度较快或出血量较多。
 2.  堵塞风险：血块可能堵塞尿道，导致急性尿潴留。患者会感到膀胱极度胀痛却无法排尿，这是泌尿外科急症，需要立即插尿管引流并冲洗膀胱。
 3.  贫血风险：持续或大量的失血可能导致急性或慢性贫血，出现头晕、乏力、心慌、面色苍白等症状，严重时会危及生命。
 4.  病情进展的信号：在已知的膀胱癌患者中，突发大量血尿可能提示肿瘤正在快速生长、表面坏死破溃，或侵犯到了血管丰富的区域。
-第二部分：正确的紧急处理与止血方法（该做什么，不该做什么）
+ 第二部分：正确的紧急处理与止血方法（该做什么，不该做什么）
 【重要警告】切勿自行使用止血药或偏方，以免延误病情或造成其他风险。
-第一步：立即就医，刻不容缓
+ 第一步：立即就医，刻不容缓
 去哪：立即前往最近医院的急诊科，或直接联系您的主治医生。告知情况后，通常会被建议去急诊。
 挂什么科：急诊科会进行初步处理，并请泌尿外科医生紧急会诊。
-第二步：医院的标准处理流程（您需要了解的）
+ 第二步：医院的标准处理流程（您需要了解的）
 医生会按以下步骤进行专业处理，目的是快速止血、解除梗阻、明确原因：
 1.  紧急评估：测量生命体征（血压、心率），查血常规看贫血程度。
 2.  解除梗阻（最优先）：
-如果患者无法排尿，医生会立即插入三腔导尿管。
-用无菌生理盐水持续冲洗膀胱，将膀胱内的血块冲洗出来，保持尿管通畅，防止新血块形成堵塞。这是最直接有效的“止血”和缓解症状的方法。
+    如果患者无法排尿，医生会立即插入三腔导尿管。
+    用无菌生理盐水持续冲洗膀胱，将膀胱内的血块冲洗出来，保持尿管通畅，防止新血块形成堵塞。这是最直接有效的“止血”和缓解症状的方法。
 3.  药物止血：
-医生可能会通过尿管向膀胱内灌注止血药物（如凝血酶、去甲肾上腺素冰盐水等），进行局部止血。
-根据情况，可能会静脉输注全身性止血药。
+    医生可能会通过尿管向膀胱内灌注止血药物（如凝血酶、去甲肾上腺素冰盐水等），进行局部止血。
+    根据情况，可能会静脉输注全身性止血药。
 4.  紧急检查和治疗：
-膀胱镜检查：在冲洗干净后，如果病情允许，医生可能会进行急诊膀胱镜检，以明确出血点。如果是肿瘤出血，有时可以在镜下进行电凝止血。
-输血：如果血红蛋白下降严重，出现失血性休克风险，会立即安排输血。
+    膀胱镜检查：在冲洗干净后，如果病情允许，医生可能会进行急诊膀胱镜检，以明确出血点。如果是肿瘤出血，有时可以在镜下进行电凝止血。
+    输血：如果血红蛋白下降严重，出现失血性休克风险，会立即安排输血。
 5.  后续根本性治疗：
-急性出血控制后，医生会根据病因制定下一步方案。如果是肿瘤引起的，可能会安排尽早手术（如根治性膀胱切除术），或进行介入栓塞治疗（通过血管造影找到给肿瘤供血的动脉并将其堵塞），这是控制顽固性血尿非常有效的方法。也可能在情况稳定后，尽快进行放疗以控制肿瘤出血。 在家等待或前往医院途中可以做的（辅助措施）
+    急性出血控制后，医生会根据病因制定下一步方案。如果是肿瘤引起的，可能会安排尽早手术（如根治性膀胱切除术），或进行介入栓塞治疗（通过血管造影找到给肿瘤供血的动脉并将其堵塞），这是控制顽固性血尿非常有效的方法。也可能在情况稳定后，尽快进行放疗以控制肿瘤出血。 在家等待或前往医院途中可以做的（辅助措施）
 绝对卧床休息，减少活动，尤其是避免腹部用力。大量饮水：如果还能排尿，多喝水、勤排尿有助于稀释血液、冲刷尿道，防止小血块形成堵塞。但若已无法排尿，则不要再喝水，以免加重膀胱胀痛。
 记录情况：注意观察尿的颜色（鲜红、暗红）、血块的大小和数量、排尿是否费力、有无腹痛腹胀，这些信息对医生非常重要。准备资料：带上以往所有的病历、CT/MRI片子、病理报告等。
-总结：请牢记以下要点
+ 总结：请牢记以下要点
 1.  膀胱癌患者出现大量血尿伴血块，是急症，有堵塞尿道的危险。
 2.  最快速有效的“止血”方法是去医院插尿管并冲洗膀胱，这不是家庭能处理的。
 3.  目标是：先通过急诊处理解决急性梗阻和出血，再针对肿瘤本身制定根本性治疗方案。
@@ -3291,8 +3286,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌患者尿血有血块，是不是很严重？怎么快速止血？
-膀胱癌患者尿血且伴有血块，通常提示病情相对严重，需尽快就医处理，不可自行盲目止血。以下是具体分析和应对原则：
+          <t>膀胱癌患者尿血且伴有血块，通常提示病情相对严重，需尽快就医处理，不可自行盲目止血。以下是具体分析和应对原则：
 一、 尿血伴血块的严重性判断
 出现血块说明出血量较大或出血速度较快，血液在膀胱内凝集形成血块，背后的原因往往反映病情进展：
 肿瘤相关因素
@@ -3352,28 +3346,27 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌患者尿血有血块，是不是很严重？怎么快速止血？
-严重性判断
+          <t>严重性判断
 出现血尿伴血块提示膀胱内出血较明显，但对严重程度不能只看“有没有血块”。膀胱癌的严重程度主要取决于肿瘤大小、数量、是否合并原位癌（CIS）、恶性程度及是否侵犯肌层（T分期）；此外，血块常因尿液在膀胱内滞留而形成，并不等同于肿瘤“更晚期”。需要强调的是，膀胱癌典型表现之一就是全程性无痛肉眼血尿，出现血块时应尽快就医评估与处理。
 需要立即就医的危险信号
-• 持续或反复出现大量鲜红尿/血块，或出现排尿困难、尿潴留（血块堵塞尿道）。
-• 伴有头晕、心悸、面色苍白、心率加快、血压下降等疑似失血表现，或血红蛋白持续下降。
-• 明显腰腹部疼痛、发热寒战，或短期内体重明显下降。
+持续或反复出现大量鲜红尿/血块，或出现排尿困难、尿潴留（血块堵塞尿道）。  
+伴有头晕、心悸、面色苍白、心率加快、血压下降等疑似失血表现，或血红蛋白持续下降。  
+明显腰腹部疼痛、发热寒战，或短期内体重明显下降。  
 出现以上任一情况，建议立即前往急诊泌尿外科处理。
 快速止血的处理路径（按轻重分级）
-• 轻度出血（偶发血块、无明显排尿困难）
-• 增加口服补液/饮水，避免憋尿；尽快联系医生评估是否短期使用止血药（如氨甲环酸、血凝酶等）或抗炎止血处理。
-• 中度出血（反复血块、颜色较深）
-• 医院行留置导尿管持续膀胱冲洗，必要时膀胱内灌注止血药，尽快膀胱镜下电灼/激光止血；若证实为肿瘤出血，可同步行经尿道肿瘤切除/电切（TURBT）以控制出血源。
-• 重度/难控出血（持续大量出血、冲洗仍鲜红、Hb下降）
-• 急诊行麻醉下膀胱镜血块清除+电凝止血；若仍难控制，转介介入放射科行膀胱动脉栓塞；极少数需开放手术止血。
-• 同步支持治疗
-• 监测血红蛋白与生命体征，必要时输血；评估并纠正凝血功能异常与抗凝/抗血小板药物使用。
+轻度出血（偶发血块、无明显排尿困难）  
+增加口服补液/饮水，避免憋尿；尽快联系医生评估是否短期使用止血药（如氨甲环酸、血凝酶等）或抗炎止血处理。  
+中度出血（反复血块、颜色较深）  
+医院行留置导尿管持续膀胱冲洗，必要时膀胱内灌注止血药，尽快膀胱镜下电灼/激光止血；若证实为肿瘤出血，可同步行经尿道肿瘤切除/电切（TURBT）以控制出血源。  
+重度/难控出血（持续大量出血、冲洗仍鲜红、Hb下降）  
+急诊行麻醉下膀胱镜血块清除+电凝止血；若仍难控制，转介介入放射科行膀胱动脉栓塞；极少数需开放手术止血。  
+同步支持治疗  
+监测血红蛋白与生命体征，必要时输血；评估并纠正凝血功能异常与抗凝/抗血小板药物使用。  
 上述措施应由泌尿外科与介入放射科协作完成，越早干预越有利于止血与降低并发症。
 就医前后注意事项
-• 不要自行反复服用阿司匹林/布洛芬等NSAIDs等可能影响凝血的药物；如正在服用抗凝/抗血小板药（如华法林、利伐沙班、氯吡格雷、阿司匹林），务必尽快联系医生评估是否需临时调整。
-• 就医前尽量多饮水有助于稀释尿液与排出血块，但若已出现排尿困难/尿潴留，不要强行用力排尿，避免加重出血或诱发膀胱痉挛。
-• 尽快完成尿常规、泌尿系超声/CT、膀胱镜等检查，明确病因与出血部位，为后续治疗（手术/介入/药物）提供依据。
+不要自行反复服用阿司匹林/布洛芬等NSAIDs等可能影响凝血的药物；如正在服用抗凝/抗血小板药（如华法林、利伐沙班、氯吡格雷、阿司匹林），务必尽快联系医生评估是否需临时调整。  
+就医前尽量多饮水有助于稀释尿液与排出血块，但若已出现排尿困难/尿潴留，不要强行用力排尿，避免加重出血或诱发膀胱痉挛。  
+尽快完成尿常规、泌尿系超声/CT、膀胱镜等检查，明确病因与出血部位，为后续治疗（手术/介入/药物）提供依据。
 医疗提示：以上为健康科普与急救要点，不能替代个体化诊疗。膀胱癌伴血尿与血块可能提示活动性出血，请尽快至泌尿外科急诊评估并按上述路径处理，避免延误最佳止血时机。</t>
         </is>
       </c>
@@ -3406,29 +3399,28 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>得了膀胱癌能活多久？
-核心决定因素：
+          <t>核心决定因素：
 1. 肿瘤分期（TNM分期）：这是最重要的因素，指肿瘤侵犯的深度。
-非肌层浸润性膀胱癌（NMIBC，占约75%）：肿瘤局限于膀胱黏膜层或黏膜下层，未侵犯肌肉层。
-预后：非常好。通过经尿道膀胱肿瘤电切术（TURBT）加上术后膀胱灌注治疗，多数患者可以长期存活，5年生存率超过90%。但主要风险是复发，需要终身定期复查膀胱镜。
-肌层浸润性膀胱癌（MIBC）：肿瘤已经侵犯膀胱肌肉层。
-预后：更具挑战性。需要积极治疗，如根治性膀胱切除术（切除整个膀胱）或综合放化疗。5年生存率根据是否发生远处转移而有很大差异，大约在40%-60%左右（局限性疾病）。
-转移性膀胱癌：癌症已扩散到膀胱以外的淋巴结或远处器官（如肺、肝、骨）。
-预后：治疗目标是控制病情、延长生存、提高生活质量。随着新型疗法出现，生存期已显著延长。中位生存期（一半患者生存的时间）从过去的不到1年，现在通过免疫治疗、靶向治疗等可延长至2年甚至更久，部分患者对治疗反应好能存活更长时间。
+   非肌层浸润性膀胱癌（NMIBC，占约75%）：肿瘤局限于膀胱黏膜层或黏膜下层，未侵犯肌肉层。
+   预后：非常好。通过经尿道膀胱肿瘤电切术（TURBT）加上术后膀胱灌注治疗，多数患者可以长期存活，5年生存率超过90%。但主要风险是复发，需要终身定期复查膀胱镜。
+   肌层浸润性膀胱癌（MIBC）：肿瘤已经侵犯膀胱肌肉层。
+   预后：更具挑战性。需要积极治疗，如根治性膀胱切除术（切除整个膀胱）或综合放化疗。5年生存率根据是否发生远处转移而有很大差异，大约在40%-60%左右（局限性疾病）。
+   转移性膀胱癌：癌症已扩散到膀胱以外的淋巴结或远处器官（如肺、肝、骨）。
+   预后：治疗目标是控制病情、延长生存、提高生活质量。随着新型疗法出现，生存期已显著延长。中位生存期（一半患者生存的时间）从过去的不到1年，现在通过免疫治疗、靶向治疗等可延长至2年甚至更久，部分患者对治疗反应好能存活更长时间。
 2.  肿瘤分级：
-低级别肿瘤：生长缓慢，侵袭性低，预后好。
-高级别肿瘤：生长快，侵袭性强，更容易进展和复发，预后相对较差。
+       低级别肿瘤：生长缓慢，侵袭性低，预后好。
+       高级别肿瘤：生长快，侵袭性强，更容易进展和复发，预后相对较差。
 3.  病理类型：
-最常见的尿路上皮癌（移行细胞癌）预后相对较好。其他类型如鳞癌、腺癌或小细胞癌等，可能更具侵袭性。
+      最常见的尿路上皮癌（移行细胞癌）预后相对较好。其他类型如鳞癌、腺癌或小细胞癌等，可能更具侵袭性。
 其他重要因素：
-患者年龄和整体健康状况：身体状况好的患者更能耐受手术和放化疗，预后通常更好。
-对治疗的反应：手术是否彻底，化疗、放疗或免疫治疗是否有效。
-是否按时随访：膀胱癌（尤其是非肌层浸润型）复发率高，严格的定期复查（膀胱镜、影像学检查）至关重要，可以早期发现并处理复发。
+   患者年龄和整体健康状况：身体状况好的患者更能耐受手术和放化疗，预后通常更好。
+   对治疗的反应：手术是否彻底，化疗、放疗或免疫治疗是否有效。
+   是否按时随访：膀胱癌（尤其是非肌层浸润型）复发率高，严格的定期复查（膀胱镜、影像学检查）至关重要，可以早期发现并处理复发。
 总结与重要建议：
 请不要被“癌症”这个词吓倒，膀胱癌，特别是早期发现的膀胱癌，是一种治疗效果相对较好的恶性肿瘤。
 1.  立即与您的医疗团队深入沟通：明确您的具体分期（TNM）、分级、病理类型。这是所有讨论的基础。
@@ -3474,8 +3466,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>得了膀胱癌能活多久
-"1. 肿瘤分期是影响生存期的核心因素
+          <t>1. 肿瘤分期是影响生存期的核心因素
 膀胱癌的分期通常采用 TNM 分期系统，反映肿瘤浸润深度、淋巴结转移和远处转移情况，不同分期的 5 年生存率差异显著：
 Ta 期、T1 期（非肌层浸润性膀胱癌）：肿瘤局限在膀胱黏膜层或黏膜下层，没有侵犯到肌层，是膀胱癌中预后较好的类型。
 经过规范治疗（如经尿道膀胱肿瘤电切术 + 术后膀胱灌注化疗），5 年生存率可达 70%～90%，部分患者可以长期生存。但这类肿瘤的复发率相对较高，需要长期随访。
@@ -3527,8 +3518,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>得了膀胱癌能活多久？
-膀胱癌生存期概览
+          <t>膀胱癌生存期概览
 生存年限差异很大，核心取决于肿瘤的分期、分级、病理类型以及治疗方式与全身状况。总体上，早期患者经规范治疗可获得长期生存，甚至达到临床治愈；而晚期/转移性患者预后明显较差。不同研究人群与统计口径会导致数值存在差异，以下为临床常见范围，供参考。
 不同分期的典型生存数据
 分期/情形     典型治疗 5年生存率或中位生存 说明
@@ -3538,16 +3528,16 @@
 远处转移（M1） 系统治疗（化疗/免疫治疗等） 5年生存率&lt;20%；1年生存率&lt;10%；平均仅数月 以延长生存与改善生活质量为主
 以上为总体区间，个体差异明显，需结合病理与随访评估。
 影响生存的关键因素
-• 病理类型与分级：如非肌层浸润性通常预后优于肌层浸润性；分级越高，复发与进展风险越大。
-• 分期与是否转移：是否累及肌层、淋巴结或远处器官是决定性变量。
-• 治疗是否规范与完整：是否完成TURBT+灌注、是否行根治性膀胱切除+淋巴结清扫、是否按时进行辅助化疗/免疫治疗等。
-• 复发与进展：NMIBC复发率可达50%–70%，少数会进展为MIBC；根治术后约有50%出现复发或转移（局部约10%–30%，其余为远处）。
-• 全身与合并症：年龄、体能状态、营养、吸烟状况与治疗耐受性会影响结局。
+病理类型与分级：如非肌层浸润性通常预后优于肌层浸润性；分级越高，复发与进展风险越大。  
+分期与是否转移：是否累及肌层、淋巴结或远处器官是决定性变量。  
+治疗是否规范与完整：是否完成TURBT+灌注、是否行根治性膀胱切除+淋巴结清扫、是否按时进行辅助化疗/免疫治疗等。  
+复发与进展：NMIBC复发率可达50%–70%，少数会进展为MIBC；根治术后约有50%出现复发或转移（局部约10%–30%，其余为远处）。  
+全身与合并症：年龄、体能状态、营养、吸烟状况与治疗耐受性会影响结局。  
 延长生存的做法
-• 早诊早治：出现无痛性肉眼血尿等警示症状应尽快就医，完善影像与内镜评估，明确分期分级后制定个体化方案。
-• 规范治疗路径：NMIBC行TURBT+术后膀胱灌注；MIBC评估后行根治性膀胱切除±辅助系统治疗；转移性病例以系统治疗为主，必要时联合局部治疗。
-• 严密随访：按医嘱定期复查（如膀胱镜、影像与尿细胞学），早期发现复发/转移并及时处理。
-• 生活方式与支持治疗：戒烟、均衡饮食、适量运动、规律作息，有助于提升治疗耐受与恢复。
+早诊早治：出现无痛性肉眼血尿等警示症状应尽快就医，完善影像与内镜评估，明确分期分级后制定个体化方案。  
+规范治疗路径：NMIBC行TURBT+术后膀胱灌注；MIBC评估后行根治性膀胱切除±辅助系统治疗；转移性病例以系统治疗为主，必要时联合局部治疗。  
+严密随访：按医嘱定期复查（如膀胱镜、影像与尿细胞学），早期发现复发/转移并及时处理。  
+生活方式与支持治疗：戒烟、均衡饮食、适量运动、规律作息，有助于提升治疗耐受与恢复。  
 重要说明
 以上为健康科普信息，不能替代医生面诊与个体化诊疗。具体预后需结合您的病理报告、分期分级、手术与随访记录由专科医生综合评估；如正接受治疗或准备制定方案，请遵循专业医嘱。</t>
         </is>
@@ -3581,23 +3571,22 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>5.膀胱癌复发率高吗？怎么预防复发？
-这是一个至关重要的问题，也是所有膀胱癌患者和医生在治疗后会持续关注的核心。直接回答您：
+          <t>这是一个至关重要的问题，也是所有膀胱癌患者和医生在治疗后会持续关注的核心。直接回答您：
 膀胱癌的复发率确实比较高，尤其是非肌层浸润性膀胱癌，但复发不等于扩散或无法控制。 通过一套科学、系统的预防策略，可以显著降低复发风险，实现长期“无瘤生存”。
 下面我将详细解释复发率和具体的预防方法。
 一、膀胱癌复发率高吗？
 答案是：取决于初始肿瘤的类型和风险分级。
 1.非肌层浸润性膀胱癌（NMIBC，占初诊患者的75%）：
-复发率很高：术后5年内复发率在 30%-80% 之间。
-为什么高？ 这是因为膀胱的尿路上皮接触相同的致癌环境（称为“场效应”），并且手术（TURBT）只能切除肉眼可见的肿瘤，无法清除微观的、不可见的“种子”细胞。
-关键点：复发大多仍然是非浸润性的，可以通过再次微创手术和灌注治疗有效控制。高复发率 ≠ 高死亡率。
+  复发率很高：术后5年内复发率在 30%-80% 之间。
+  为什么高？ 这是因为膀胱的尿路上皮接触相同的致癌环境（称为“场效应”），并且手术（TURBT）只能切除肉眼可见的肿瘤，无法清除微观的、不可见的“种子”细胞。
+  关键点：复发大多仍然是非浸润性的，可以通过再次微创手术和灌注治疗有效控制。高复发率 ≠ 高死亡率。
 2.肌层浸润性膀胱癌（MIBC）：
-经过根治性膀胱切除术后，局部复发率相对较低（约10%-20%），但远处转移（如肺、肝、骨）的风险更高，是影响生存的主要威胁。
+  经过根治性膀胱切除术后，局部复发率相对较低（约10%-20%），但远处转移（如肺、肝、骨）的风险更高，是影响生存的主要威胁。
 总结： 对于占大多数的NMIBC患者，“与复发共存，并有效管理它”是长期治疗的主题。
 二、如何预防复发？（三位一体的核心策略）
 预防复发是一个需要医患紧密配合、长期坚持的系统工程。核心策略包括：
@@ -3606,7 +3595,7 @@
 1.膀胱镜检查：金标准。术后前2年，通常每3-6个月一次；2-5年内，每6-12个月一次；5年后每年一次。医生直接用镜子观察膀胱内壁，是最直接的方法。
 2.尿脱落细胞学检查：检查尿液中是否有癌细胞。
 3.影像学检查：如泌尿系统B超、CT尿路成像（CTU），用于检查上尿路（肾、输尿管）有无肿瘤，以及有无远处转移。
-必须遵医嘱：绝不能因为感觉良好或害怕检查而中断复查。
+   必须遵医嘱：绝不能因为感觉良好或害怕检查而中断复查。
 第二支柱：规范的术后辅助治疗（降低风险）
 主要针对NMIBC患者，手术后立即开始。
 1.术后膀胱灌注治疗：
@@ -3617,9 +3606,9 @@
 1.彻底戒烟：这是最重要、最有效的措施！ 吸烟是膀胱癌的首要危险因素，持续吸烟会使复发风险翻倍甚至更高。
 2.大量饮水：每天保证2升以上的饮水量（心肾功能正常者）。充足饮水能稀释尿液中的致癌物，减少其与膀胱黏膜的接触时间和浓度。
 3.均衡饮食：
-多摄入：新鲜蔬菜水果（特别是富含抗氧化剂的十字花科蔬菜、番茄、浆果等）。
-限制：红肉和加工肉类（火腿、香肠等）。
-避免：可能含有害物质的食物。
+  多摄入：新鲜蔬菜水果（特别是富含抗氧化剂的十字花科蔬菜、番茄、浆果等）。
+  限制：红肉和加工肉类（火腿、香肠等）。
+  避免：可能含有害物质的食物。
 4.避免职业暴露：如果工作中接触染料、化工品等，务必做好职业防护。
 5.谨慎使用药物：长期服用某些镇痛药（如非那西丁）可能增加风险，用药需咨询医生。
 总结与心态调整
@@ -3664,8 +3653,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌复发率高吗？怎么预防复发？
-"膀胱癌的复发率相对较高，尤其是非肌层浸润性膀胱癌，这也是膀胱癌治疗后需要长期随访的核心原因。预防复发需要从术后规范治疗、生活方式调整、定期复查三个维度综合干预。
+          <t>膀胱癌的复发率相对较高，尤其是非肌层浸润性膀胱癌，这也是膀胱癌治疗后需要长期随访的核心原因。预防复发需要从术后规范治疗、生活方式调整、定期复查三个维度综合干预。
 一、 膀胱癌的复发率情况
 膀胱癌的复发率和肿瘤分期、分级密切相关：
 非肌层浸润性膀胱癌（Ta、T1 期）
@@ -3686,7 +3674,7 @@
 定期复查，早发现早处理
 复发的肿瘤早期处理预后较好，因此复查是预防复发的重要环节：
 非肌层浸润性膀胱癌：术后前 2 年每 3 个月复查一次膀胱镜；第 3～5 年每 6 个月复查一次；5 年后每年复查一次。同时定期做尿常规、泌尿系超声检查。
-肌层浸润性膀胱癌：术后前 2 年每 3 个月复查一次腹部 / 盆腔 CT、尿常规、肿瘤标志物等；之后根据病情调整复查频率，警惕远处转移。"</t>
+肌层浸润性膀胱癌：术后前 2 年每 3 个月复查一次腹部 / 盆腔 CT、尿常规、肿瘤标志物等；之后根据病情调整复查频率，警惕远处转移。</t>
         </is>
       </c>
     </row>
@@ -3723,8 +3711,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌复发率高吗？怎么预防复发？
-膀胱癌的复发率相对较高，尤其是非肌层浸润性膀胱癌（NMIBC）。
+          <t>膀胱癌的复发率相对较高，尤其是非肌层浸润性膀胱癌（NMIBC）。
 具体来说：
 非肌层浸润性膀胱癌（NMIBC）：复发率较高，据报道，大约50%-70%的患者在治疗后的几年内会出现复发。部分患者还可能进展为肌层浸润性膀胱癌。
 肌层浸润性膀胱癌（MIBC）：根治性手术后，大约有50%的患者会出现复发或转移，其中局部复发约占10%-30%，远处转移则更为常见。
@@ -3782,13 +3769,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>9.膀胱癌容易骨转移吗？
-这是一个非常重要的问题。总的来说，与肺癌、乳腺癌、前列腺癌相比，膀胱癌发生骨转移的几率相对较低，但确实会发生，尤其是在晚期或高级别肿瘤中。
+          <t>这是一个非常重要的问题。总的来说，与肺癌、乳腺癌、前列腺癌相比，膀胱癌发生骨转移的几率相对较低，但确实会发生，尤其是在晚期或高级别肿瘤中。
 下面是详细的分析：
 1. 总体转移规律与常见部位
 膀胱癌最常见的转移途径是 淋巴转移 和 血行转移。
@@ -3802,28 +3788,28 @@
 3. 骨转移的特点和常见部位
 常见部位：膀胱癌骨转移最常发生在 中轴骨，如脊柱（特别是胸椎和腰椎）、骨盆、肋骨。这些部位血供丰富，癌细胞容易“定居”。
 症状：骨转移可能引起：
-疼痛：持续、进行性加重的骨痛，夜间尤甚，休息不缓解。
-病理性骨折：骨质被破坏后，轻微外力甚至日常活动即可导致骨折。
-脊髓压迫：如果转移灶在脊柱，可能压迫脊髓，导致背部剧痛、下肢无力、麻木，甚至大小便失禁，这是肿瘤急症，需立即处理。
-高钙血症：骨质破坏导致血钙升高，可引起恶心、呕吐、嗜睡、意识模糊等。
+    疼痛：持续、进行性加重的骨痛，夜间尤甚，休息不缓解。
+    病理性骨折：骨质被破坏后，轻微外力甚至日常活动即可导致骨折。
+    脊髓压迫：如果转移灶在脊柱，可能压迫脊髓，导致背部剧痛、下肢无力、麻木，甚至大小便失禁，这是肿瘤急症，需立即处理。
+    高钙血症：骨质破坏导致血钙升高，可引起恶心、呕吐、嗜睡、意识模糊等。
 4. 如何发现和诊断骨转移？
 影像学检查：
-全身骨扫描：是筛查骨转移最常用的初步手段，灵敏度高。
-CT或MRI：对特定疼痛部位进行CT或MRI扫描，可以更清晰地显示骨质破坏的细节和软组织侵犯情况。
-PETCT：在评估全身转移（包括骨转移）方面更精确，能同时显示代谢活性，但价格昂贵。
+    全身骨扫描：是筛查骨转移最常用的初步手段，灵敏度高。
+    CT或MRI：对特定疼痛部位进行CT或MRI扫描，可以更清晰地显示骨质破坏的细节和软组织侵犯情况。
+    PETCT：在评估全身转移（包括骨转移）方面更精确，能同时显示代谢活性，但价格昂贵。
 确诊：有时需要通过骨穿刺活检取得病理，以最终确诊是否为膀胱癌转移。
 5. 发生骨转移后的治疗
 一旦发生骨转移，意味着疾病进入晚期（IV期），治疗目标是控制病情、缓解症状、提高生活质量、延长生存期。治疗是综合性的：
 1.  全身治疗：
-化疗：仍是基础治疗方案。
-免疫治疗（PD1/PDL1抑制剂）：如帕博利珠单抗、阿替利珠单抗等，已成为晚期膀胱癌的重要选择。
-抗体药物偶联物：如恩诺单抗、戈沙妥珠单抗，用于化疗和免疫治疗失败后的患者。
-靶向治疗：针对特定基因突变（如FGFR）的患者。
+    化疗：仍是基础治疗方案。
+    免疫治疗（PD1/PDL1抑制剂）：如帕博利珠单抗、阿替利珠单抗等，已成为晚期膀胱癌的重要选择。
+    抗体药物偶联物：如恩诺单抗、戈沙妥珠单抗，用于化疗和免疫治疗失败后的患者。
+    靶向治疗：针对特定基因突变（如FGFR）的患者。
 2.  针对骨转移的局部治疗：
-双膦酸盐或地舒单抗：每月一次的注射，可强效抑制骨破坏、减少骨骼相关事件（如骨折）、缓解骨痛，是骨转移的标准治疗药物。
-局部放疗：对疼痛剧烈的骨转移灶进行外照射放疗，是缓解骨痛非常有效的方法。
-手术：如果发生或即将发生病理性骨折、脊柱不稳定或脊髓压迫，可能需要骨科手术进行固定或减压。
-止痛治疗：根据疼痛程度，规范使用止痛药（从非甾体抗炎药到阿片类药物）。
+    双膦酸盐或地舒单抗：每月一次的注射，可强效抑制骨破坏、减少骨骼相关事件（如骨折）、缓解骨痛，是骨转移的标准治疗药物。
+    局部放疗：对疼痛剧烈的骨转移灶进行外照射放疗，是缓解骨痛非常有效的方法。
+    手术：如果发生或即将发生病理性骨折、脊柱不稳定或脊髓压迫，可能需要骨科手术进行固定或减压。
+    止痛治疗：根据疼痛程度，规范使用止痛药（从非甾体抗炎药到阿片类药物）。
 总结膀胱癌会发生骨转移，虽然不是最高发，但在晚期患者中较为常见。
 其风险与肿瘤分期、分级和淋巴结状态密切相关。
 骨转移的主要症状是骨痛，严重时可导致骨折和脊髓压迫等急症。
@@ -3865,8 +3851,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>9.膀胱癌容易骨转移吗？
-"膀胱癌有可能发生骨转移，但它不属于膀胱癌最常见的转移部位，骨转移更多见于晚期、高级别或肌层浸润性膀胱癌患者。
+          <t>膀胱癌有可能发生骨转移，但它不属于膀胱癌最常见的转移部位，骨转移更多见于晚期、高级别或肌层浸润性膀胱癌患者。
 1. 膀胱癌转移的常见路径与部位
 膀胱癌的转移主要通过淋巴转移和血行转移：
 淋巴转移：是膀胱癌较早出现的转移方式，常见转移部位是盆腔淋巴结。
@@ -3883,7 +3868,7 @@
 影像学检查：全身骨扫描（ECT） 是筛查骨转移的首选方法，敏感度较高；若发现可疑病灶，会进一步做CT 或磁共振（MRI） 明确诊断。
 肿瘤标志物：部分患者的碱性磷酸酶（ALP）水平可能升高，可作为辅助参考指标。
 总结
-膀胱癌并不轻易发生骨转移，骨转移属于疾病晚期的表现之一。对于早中期膀胱癌患者，骨转移的风险较低，无需过度担心；而晚期患者则需要遵医嘱定期排查，以便早发现、早干预，减轻症状、延长生存期。"</t>
+膀胱癌并不轻易发生骨转移，骨转移属于疾病晚期的表现之一。对于早中期膀胱癌患者，骨转移的风险较低，无需过度担心；而晚期患者则需要遵医嘱定期排查，以便早发现、早干预，减轻症状、延长生存期。</t>
         </is>
       </c>
     </row>
@@ -3920,20 +3905,19 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌容易骨转移吗
-膀胱癌发生骨转移的概率相对低于肺癌、乳腺癌、前列腺癌等，但在特定情况下仍可能发生，尤其是当肿瘤进展到晚期时。
+          <t>膀胱癌发生骨转移的概率相对低于肺癌、乳腺癌、前列腺癌等，但在特定情况下仍可能发生，尤其是当肿瘤进展到晚期时。
 具体来说：
 1.  整体概率：膀胱癌患者中，发生骨转移的比例相对较低，大约在5% - 15%左右。大多数膀胱癌患者在确诊时或疾病发展过程中，首先出现的转移部位往往是盆腔淋巴结、肺部、肝脏等。
 2.  易发生骨转移的膀胱癌类型：
-◦   晚期膀胱癌：当膀胱癌发展到晚期（通常是IV期），肿瘤细胞可以通过血液循环扩散到骨骼。
-◦   特定的病理类型：某些特殊类型的膀胱癌，如鳞状细胞癌、腺癌或小细胞癌，相对于最常见的尿路上皮癌，可能更容易发生远处转移，包括骨转移。
-◦   侵袭性强的肿瘤：肿瘤分级高、分期晚、增殖快、侵袭性强的膀胱癌，发生转移的风险更高。
+    ◦   晚期膀胱癌：当膀胱癌发展到晚期（通常是IV期），肿瘤细胞可以通过血液循环扩散到骨骼。
+    ◦   特定的病理类型：某些特殊类型的膀胱癌，如鳞状细胞癌、腺癌或小细胞癌，相对于最常见的尿路上皮癌，可能更容易发生远处转移，包括骨转移。
+    ◦   侵袭性强的肿瘤：肿瘤分级高、分期晚、增殖快、侵袭性强的膀胱癌，发生转移的风险更高。
 3.  骨转移的常见部位：如果发生骨转移，常见于脊柱、骨盆、肋骨、股骨等部位。
 4.  骨转移的症状：
-◦   疼痛：这是最常见的症状，通常为持续性钝痛或酸痛，夜间或活动时加重。
-◦   病理性骨折：骨骼被癌细胞破坏后变得脆弱，轻微外力即可导致骨折。
-◦   神经压迫症状：如果转移到脊柱，可能压迫脊髓或神经根，导致肢体麻木、无力、大小便失禁等。
-◦   高钙血症：骨转移灶释放过多的钙离子进入血液，可引起恶心、呕吐、便秘、多尿、口渴、意识模糊等症状。
+    ◦   疼痛：这是最常见的症状，通常为持续性钝痛或酸痛，夜间或活动时加重。
+    ◦   病理性骨折：骨骼被癌细胞破坏后变得脆弱，轻微外力即可导致骨折。
+    ◦   神经压迫症状：如果转移到脊柱，可能压迫脊髓或神经根，导致肢体麻木、无力、大小便失禁等。
+    ◦   高钙血症：骨转移灶释放过多的钙离子进入血液，可引起恶心、呕吐、便秘、多尿、口渴、意识模糊等症状。
 总结一下：膀胱癌骨转移的发生率不高，但并非完全不会发生。晚期膀胱癌、侵袭性强的肿瘤以及某些特殊病理类型的膀胱癌更容易发生骨转移。如果出现不明原因的骨痛、病理性骨折或神经压迫症状，应及时就医进行检查，以排除骨转移的可能。对于膀胱癌患者，定期的随访复查非常重要，包括影像学检查（如骨扫描、CT、MRI等），以便早期发现潜在的转移病灶。</t>
         </is>
       </c>
@@ -3966,26 +3950,25 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>14.高级别浸润性膀胱癌患者，没转移的情况下能活几年？
-这是一个非常关键且患者和家属最关心的问题。首先必须强调：这是一个无法给出确切年数的预测性问题。 对于没有转移的肌层浸润性膀胱癌，医学上通常不用“能活几年”来回答，而是用5年生存率作为最重要的评估指标。
+          <t>这是一个非常关键且患者和家属最关心的问题。首先必须强调：这是一个无法给出确切年数的预测性问题。 对于没有转移的肌层浸润性膀胱癌，医学上通常不用“能活几年”来回答，而是用5年生存率作为最重要的评估指标。
 不过，我可以为您详细解析影响预后的关键因素、当前的治疗目标和可以达到的生存数据，帮助您理解“治愈”的可能性。
-核心概念：治愈是主要目标：对于没有远处转移（医学上称为 M0）的肌层浸润性膀胱癌，治疗的主要目标就是根治，即长期生存甚至治愈。这不是姑息治疗，而是追求彻底清除肿瘤。
-影响生存期的关键因素1.  病理分期（T分期）：这是最重要的因素。T2期：肿瘤侵犯膀胱肌肉层浅层。预后相对较好。T3期：肿瘤侵犯膀胱肌肉层深层或穿透膀胱壁。 T4期：肿瘤侵犯前列腺、精囊、子宫、阴道或盆壁。分期越晚，预后相对越差。
+ 核心概念：治愈是主要目标：对于没有远处转移（医学上称为 M0）的肌层浸润性膀胱癌，治疗的主要目标就是根治，即长期生存甚至治愈。这不是姑息治疗，而是追求彻底清除肿瘤。
+ 影响生存期的关键因素1.  病理分期（T分期）：这是最重要的因素。T2期：肿瘤侵犯膀胱肌肉层浅层。预后相对较好。T3期：肿瘤侵犯膀胱肌肉层深层或穿透膀胱壁。 T4期：肿瘤侵犯前列腺、精囊、子宫、阴道或盆壁。分期越晚，预后相对越差。
 2.  淋巴结状态（N分期）： N0：手术清扫的盆腔淋巴结没有癌细胞。这是预后良好的标志。
-N1N3：淋巴结有转移。即使影像学未发现远处转移，淋巴结阳性也意味着更高的复发风险，预后显著差于N0。
+   N1N3：淋巴结有转移。即使影像学未发现远处转移，淋巴结阳性也意味着更高的复发风险，预后显著差于N0。
 3. 治疗方案是否规范： 是否接受了“新辅助化疗+根治性膀胱切除术” 这一标准治疗。这是提高长期生存率的基石。手术质量：是否进行了彻底的盆腔淋巴结清扫。如果选择保膀胱治疗，对治疗的响应程度如何。
 4.  肿瘤生物学特性：是否存在某些高危分子标志物（如p53基因突变等）。
 5.  患者自身状况：年龄、体能状态、有无严重合并症（如心、肺、肾功能）等，这些会影响治疗的完成度和身体恢复能力。 基于数据的生存率参考（请理解其统计意义）
 以下是基于大型临床研究的5年生存率数据，这是目前最可靠的参考。“5年生存率”不代表只能活5年，而是指治疗后存活超过5年的患者比例，临床上常将其视为“临床治愈”的指标。总体情况（综合所有分期）：接受标准根治性膀胱切除术的肌层浸润性膀胱癌患者，5年总生存率约为50%65%。
 按病理分期细化（基于术后病理，最准确）：器官局限性疾病（pT2, N0）：这是预后最好的情况。5年生存率可达70%80%以上。很多患者可以实现长期无病生存。 局部晚期但淋巴结阴性（pT3pT4a, N0）：5年生存率约为40%60%。 淋巴结阳性（任何T, N+）：即使术前影像学未发现，术后病理证实淋巴结转移，预后会变差，5年生存率降至20%35%。但积极的术后辅助治疗（化疗/免疫治疗）可能改善这一数字。
 关键治疗的影响：  新辅助化疗的作用：对于T2期及以上患者，术前进行以顺铂为基础的化疗，可以将5年生存率绝对提高5%10%。例如，使一部分患者的生存率从50%提升至60%。
-一个重要的“希望点”：精准医学时代的新进展：过去的数据是基于传统放化疗得出的。如今，免疫治疗和靶向治疗为膀胱癌的治疗带来了新希望。免疫治疗作为辅助治疗：对于高危患者（如pT3/pT4或淋巴结阳性），术后使用帕博利珠单抗（K药） 等免疫检查点抑制剂进行辅助治疗，已被证实能显著降低复发风险，延长无病生存期。这意味着更多患者有机会实现长期治愈。未来的可能性：新的药物组合和疗法仍在不断研发中，患者的生存前景在未来有继续改善的趋势。
-总结与核心建议：不要纠结于一个具体的年数：生存数据是群体统计，每位患者都是独特的个体。积极、规范的治疗是影响结果最可控的因素。2. 治愈是现实目标：特别是对于分期较早（如T2N0）且接受标准治疗的患者，长期生存和临床治愈的可能性非常大。
+ 一个重要的“希望点”：精准医学时代的新进展：过去的数据是基于传统放化疗得出的。如今，免疫治疗和靶向治疗为膀胱癌的治疗带来了新希望。免疫治疗作为辅助治疗：对于高危患者（如pT3/pT4或淋巴结阳性），术后使用帕博利珠单抗（K药） 等免疫检查点抑制剂进行辅助治疗，已被证实能显著降低复发风险，延长无病生存期。这意味着更多患者有机会实现长期治愈。未来的可能性：新的药物组合和疗法仍在不断研发中，患者的生存前景在未来有继续改善的趋势。
+ 总结与核心建议：不要纠结于一个具体的年数：生存数据是群体统计，每位患者都是独特的个体。积极、规范的治疗是影响结果最可控的因素。2. 治愈是现实目标：特别是对于分期较早（如T2N0）且接受标准治疗的患者，长期生存和临床治愈的可能性非常大。
 3. 当前最关键的行动：寻求规范治疗：立即咨询专业的泌尿肿瘤中心，组建多学科团队，制定以 “根治”为目标的规范治疗方案（通常首选新辅助化疗+根治性手术）。完成全部治疗：尽最大努力完成计划中的手术、化疗等所有治疗环节。 坚持严密随访：治疗后的定期复查（包括影像学和膀胱镜）至关重要，以便早期发现并处理任何复发迹象。
 请与您的主治医生深入沟通，他们可以根据具体的病理报告、影像结果和您的身体状况，给出更个体化的预后分析和治疗建议。保持信心，积极配合治疗，是应对这个疾病最重要的态度。</t>
         </is>
@@ -4024,8 +4007,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>高级别浸润性膀胱癌患者，没转移的情况下能活几年？
-未发生转移的高级别肌层浸润性膀胱癌患者的生存期，主要取决于治疗方案的选择、肿瘤分期（T2/T3/T4a）以及患者的身体基础状况，总体 5 年生存率在 40%~70% 之间，具体分层如下：
+          <t>未发生转移的高级别肌层浸润性膀胱癌患者的生存期，主要取决于治疗方案的选择、肿瘤分期（T2/T3/T4a）以及患者的身体基础状况，总体 5 年生存率在 40%~70% 之间，具体分层如下：
 1. 按肿瘤分期划分的生存期
 高级别肌层浸润性膀胱癌的分期（T 分期）是影响预后的核心因素，无远处转移（M0）时的生存数据如下：
 T2 期（肿瘤侵犯浅肌层）：接受根治性膀胱全切术 + 盆腔淋巴结清扫术后，5 年生存率可达 60%~70%；若选择保留膀胱的放化疗综合方案，5 年生存率约 50%~60%，但复发率相对更高。
@@ -4088,37 +4070,36 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>高级别浸润性膀胱癌患者，没转移的情况下能活几年？
-对于高级别肌层浸润性膀胱癌（MIBC）且无转移的患者，其生存期受多种因素影响，包括肿瘤分期、分级、治疗方案、患者身体状况等。以下是基于现有医学研究和临床实践的一般性信息，供参考：
+          <t>对于高级别肌层浸润性膀胱癌（MIBC）且无转移的患者，其生存期受多种因素影响，包括肿瘤分期、分级、治疗方案、患者身体状况等。以下是基于现有医学研究和临床实践的一般性信息，供参考：
 1. 关键影响因素
-• 肿瘤分期（T分期）：
-• T2a/T2b（肿瘤侵犯肌层但未突破膀胱壁）：若接受根治性膀胱切除+淋巴结清扫+辅助化疗，5年生存率约为50%-70%。
-• T3/T4（肿瘤侵犯膀胱周围组织或邻近器官）：即使无远处转移，5年生存率可能降至30%-50%，需更积极的综合治疗。
-• 治疗方案：
-• 根治性手术+辅助化疗：是目前的标准治疗，可显著提高生存率。
-• 保膀胱综合治疗（如TMT：TURBT+同步放化疗）：在严格筛选的患者中，5年生存率与手术相当，但需密切随访。
-• 患者因素：
-• 年龄、体能状态、合并症（如心脏病、糖尿病）及治疗耐受性会影响预后。
-• 规范随访和及时干预复发/转移是延长生存的关键。
+肿瘤分期（T分期）：
+T2a/T2b（肿瘤侵犯肌层但未突破膀胱壁）：若接受根治性膀胱切除+淋巴结清扫+辅助化疗，5年生存率约为50%-70%。
+T3/T4（肿瘤侵犯膀胱周围组织或邻近器官）：即使无远处转移，5年生存率可能降至30%-50%，需更积极的综合治疗。
+治疗方案：
+根治性手术+辅助化疗：是目前的标准治疗，可显著提高生存率。
+保膀胱综合治疗（如TMT：TURBT+同步放化疗）：在严格筛选的患者中，5年生存率与手术相当，但需密切随访。
+患者因素：
+年龄、体能状态、合并症（如心脏病、糖尿病）及治疗耐受性会影响预后。
+规范随访和及时干预复发/转移是延长生存的关键。
 2. 生存数据参考
-• 5年生存率：
-• 对于T2期无转移的高级别MIBC，5年生存率约为50%-70%。
-• 对于T3/T4期无转移者，5年生存率约为30%-50%。
-• 10年生存率：
-• 随着时间推移，复发和转移风险增加，10年生存率通常低于5年生存率，具体数值因个体差异较大。
+5年生存率：
+对于T2期无转移的高级别MIBC，5年生存率约为50%-70%。
+对于T3/T4期无转移者，5年生存率约为30%-50%。
+10年生存率：
+随着时间推移，复发和转移风险增加，10年生存率通常低于5年生存率，具体数值因个体差异较大。
 3. 延长生存的措施
-• 规范治疗：
-• 尽早接受根治性膀胱切除或保膀胱综合治疗，术后根据病理结果决定是否需辅助化疗/免疫治疗。
-• 密切随访：
-• 术后定期复查（如膀胱镜、CT/MRI、尿细胞学），早期发现复发或转移并及时处理。
-• 生活方式调整：
-• 戒烟、健康饮食、适量运动，改善整体健康状况。
-• 心理支持：
-• 保持积极心态，必要时寻求心理干预，有助于提高治疗依从性和生活质量。
+规范治疗：
+尽早接受根治性膀胱切除或保膀胱综合治疗，术后根据病理结果决定是否需辅助化疗/免疫治疗。
+密切随访：
+术后定期复查（如膀胱镜、CT/MRI、尿细胞学），早期发现复发或转移并及时处理。
+生活方式调整：
+戒烟、健康饮食、适量运动，改善整体健康状况。
+心理支持：
+保持积极心态，必要时寻求心理干预，有助于提高治疗依从性和生活质量。
 4. 重要提示
-• 以上数据为群体统计结果，个体预后差异较大，需结合具体病情、治疗方案及随访情况由医生综合评估。
-• 医学上没有绝对的“能活几年”的答案，积极治疗和管理可显著改善预后。
-• 建议患者与主治医生充分沟通，制定个性化治疗方案，并严格遵循医嘱进行随访和治疗。
+以上数据为群体统计结果，个体预后差异较大，需结合具体病情、治疗方案及随访情况由医生综合评估。
+医学上没有绝对的“能活几年”的答案，积极治疗和管理可显著改善预后。
+建议患者与主治医生充分沟通，制定个性化治疗方案，并严格遵循医嘱进行随访和治疗。
 总结：高级别MIBC无转移患者的生存期受多种因素影响，规范治疗和密切随访是提高生存率的关键。请务必在专业医生指导下进行治疗和随访，以获得最佳预后。</t>
         </is>
       </c>
@@ -4151,27 +4132,26 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>15.膀胱癌电切术后会复发吗？复发几率大概是多少？
-这是一个所有膀胱癌患者和家属都非常关心的问题。答案是：会复发。 膀胱癌，尤其是非肌层浸润性膀胱癌，一个显著的特点就是高复发率。
+          <t>这是一个所有膀胱癌患者和家属都非常关心的问题。答案是：会复发。 膀胱癌，尤其是非肌层浸润性膀胱癌，一个显著的特点就是高复发率。
 但请先不要过于焦虑，复发率的高低差异巨大，并且有非常明确的预防和治疗策略。以下是基于医学证据的详细解答：核心结论：复发率因风险分级而异，膀胱癌经尿道电切术后的复发几率不是固定的，它完全取决于术后病理确定的 “风险分级” 。医生会根据肿瘤的侵犯深度（T分期）、细胞恶性程度（分级）、是否多发、是否合并原位癌、是否复发等因素，将患者分为低危、中危、高危三个组。不同组别的复发率有显著差异。
 各风险分层的复发几率及原因
 1.  低危组
-特征：单发、Ta期（仅侵犯黏膜表层）、低级别（G1）、肿瘤直径&lt;3cm、且无复发史。
-复发几率：1年复发率约15%，5年复发率约31%。
-原因：肿瘤侵袭性低，但膀胱内环境（“土壤”）可能仍存在致癌因素，可能导致新发肿瘤。
+    特征：单发、Ta期（仅侵犯黏膜表层）、低级别（G1）、肿瘤直径&lt;3cm、且无复发史。
+    复发几率：1年复发率约15%，5年复发率约31%。
+    原因：肿瘤侵袭性低，但膀胱内环境（“土壤”）可能仍存在致癌因素，可能导致新发肿瘤。
 2.  中危组
-特征：介于低危和高危之间。例如：多发或复发的Ta期低级别肿瘤；单一的Ta期高级别肿瘤；或初发的T1期低级别肿瘤等。
-复发几率：1年复发率约24%38%，5年复发率约46%62%。
-原因：肿瘤生物学行为更具侵袭性。
+    特征：介于低危和高危之间。例如：多发或复发的Ta期低级别肿瘤；单一的Ta期高级别肿瘤；或初发的T1期低级别肿瘤等。
+    复发几率：1年复发率约24%38%，5年复发率约46%62%。
+    原因：肿瘤生物学行为更具侵袭性。
 3.  高危组（复发风险最高，需重点关注）
-特征：符合以下任一条件：T1期（侵犯黏膜下层）、高级别（G3）、合并原位癌、多发、大体积（&gt;3cm）、短期内复发。
-复发几率：1年复发率高达61%，5年复发率可超过70%80%。更重要的是，进展为肌层浸润性膀胱癌的风险也显著增高（5年约20%40%）。
-原因：肿瘤本身恶性度高，极易在切除部位或膀胱其他位置复发，并有向深处侵犯的倾向。
+    特征：符合以下任一条件：T1期（侵犯黏膜下层）、高级别（G3）、合并原位癌、多发、大体积（&gt;3cm）、短期内复发。
+    复发几率：1年复发率高达61%，5年复发率可超过70%80%。更重要的是，进展为肌层浸润性膀胱癌的风险也显著增高（5年约20%40%）。
+    原因：肿瘤本身恶性度高，极易在切除部位或膀胱其他位置复发，并有向深处侵犯的倾向。
 为什么会复发？（复发机制）
 肿瘤残留：电切可能无法完全清除肉眼不可见的微小病灶或原位癌。
 肿瘤种植：手术中脱落的癌细胞可能在其他部位的膀胱黏膜上“扎根”生长。
@@ -4228,8 +4208,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌电切术后会复发吗？复发几率大概是多少？
-膀胱癌经尿道电切术（TURBT）后存在明确的复发风险，复发几率与肿瘤的分期、分级、数量、大小及术后辅助治疗密切相关，不同人群的复发率差异显著。
+          <t>膀胱癌经尿道电切术（TURBT）后存在明确的复发风险，复发几率与肿瘤的分期、分级、数量、大小及术后辅助治疗密切相关，不同人群的复发率差异显著。
 一、 复发风险的核心分层依据
 复发率的高低主要取决于肿瘤的危险分层，临床上通常分为低危、中危、高危三类，对应的复发数据如下：
 低危非肌层浸润性膀胱癌
@@ -4291,11 +4270,10 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌电切术后会复发吗？复发几率大概是多少？
-总体结论
+          <t>总体结论
 会复发，尤其是非肌层浸润性膀胱癌（NMIBC）患者。复发风险与肿瘤的分级、分期、是否合并原位癌（CIS）、切除是否彻底以及术后是否进行膀胱内灌注等密切相关。总体上，NMIBC经经尿道膀胱肿瘤电切（TURBT）后属于“高复发”疾病谱，需要规范的术后辅助治疗与随访以降低风险与进展风险。
 复发率区间与典型数据
-• 下表为不同情境下的典型复发风险（以5年复发率为主，供参考，实际需结合个体病理与随访依从性）：
+下表为不同情境下的典型复发风险（以5年复发率为主，供参考，实际需结合个体病理与随访依从性）：
 情形 典型复发率 说明
 NMIBC（中高危）行TURBT 约24%–50% 多中心长期随访范围；是否合并CIS、切缘与是否做灌注影响显著
 NMIBC行TURBT + 术后即刻膀胱灌注化疗 复发率较不灌注者降低约14% 即刻灌注有助于清除残留肿瘤细胞
@@ -4303,17 +4281,17 @@
 肌层浸润性膀胱癌（MIBC）行TURBT（非根治） 约20%–30% 此类患者多需考虑根治性膀胱切除或保膀胱综合治疗路径
 上述区间来自临床研究与专家共识性解读，具体个体风险需结合病理分期与治疗方案评估。
 影响复发的关键因素
-• 肿瘤分级与分期：分级越高、越接近肌层，复发与进展风险越高。
-• 是否合并原位癌（CIS）：CIS提示更高复发与进展风险。
-• 切除质量：是否达到全层切除、是否存在阳性切缘。
-• 术后是否规范膀胱内治疗：如即刻/早期膀胱灌注化疗或卡介苗（BCG）。
-• 个体危险因素：如吸烟、长期接触致癌物、免疫功能低下等。
+肿瘤分级与分期：分级越高、越接近肌层，复发与进展风险越高。  
+是否合并原位癌（CIS）：CIS提示更高复发与进展风险。  
+切除质量：是否达到全层切除、是否存在阳性切缘。  
+术后是否规范膀胱内治疗：如即刻/早期膀胱灌注化疗或卡介苗（BCG）。  
+个体危险因素：如吸烟、长期接触致癌物、免疫功能低下等。  
 以上因素共同决定复发概率与随访强度。
 如何降低风险与随访建议
-• 术后尽早进行膀胱内灌注（化疗或BCG，由病理与风险分层决定），并按时完成维持治疗，可显著降低复发风险。
-• 按风险分层进行规律膀胱镜随访：术后前2年每约3个月复查一次；若2年内无复发，可改为每6个月；5年后仍未复发可每年一次；若10年未复发，通常不再常规膀胱镜，改为定期B超等影像随访。
-• 出现无痛性肉眼血尿、尿频尿急尿痛、夜尿增多等提示复发或并发症的信号，应尽快就医复查。
-• 生活方式干预：戒烟、避免接触致癌物、规律作息与适量运动，有助于提高治疗耐受与降低复发风险。
+术后尽早进行膀胱内灌注（化疗或BCG，由病理与风险分层决定），并按时完成维持治疗，可显著降低复发风险。  
+按风险分层进行规律膀胱镜随访：术后前2年每约3个月复查一次；若2年内无复发，可改为每6个月；5年后仍未复发可每年一次；若10年未复发，通常不再常规膀胱镜，改为定期B超等影像随访。  
+出现无痛性肉眼血尿、尿频尿急尿痛、夜尿增多等提示复发或并发症的信号，应尽快就医复查。  
+生活方式干预：戒烟、避免接触致癌物、规律作息与适量运动，有助于提高治疗耐受与降低复发风险。
 医疗提示
 以上为健康科普信息，不能替代个体化医疗建议。具体复发风险与随访方案需由泌尿外科/肿瘤科结合您的病理报告、分期与治疗方案综合评估与制定。</t>
         </is>
@@ -4347,17 +4325,16 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>6.膀胱癌术后灌注治疗有什么副作用？要注意什么？
-膀胱癌术后膀胱灌注治疗是预防非肌层浸润性膀胱癌（NMIBC）复发和进展的关键手段。了解其副作用和注意事项，可以帮助您更好地配合治疗、减轻不适，并确保治疗安全有效。
+          <t>膀胱癌术后膀胱灌注治疗是预防非肌层浸润性膀胱癌（NMIBC）复发和进展的关键手段。了解其副作用和注意事项，可以帮助您更好地配合治疗、减轻不适，并确保治疗安全有效。
 灌注治疗主要分为两种：化疗药物灌注（如丝裂霉素、表柔比星、吉西他滨等）和免疫药物灌注（主要是卡介苗，BCG）。它们的副作用有所不同。
-一、常见副作用（反应）
-1. 化疗药物灌注的副作用（通常较轻，以局部刺激为主）
-膀胱刺激症状（化学性膀胱炎）：最常见。
+ 一、常见副作用（反应）
+ 1. 化疗药物灌注的副作用（通常较轻，以局部刺激为主）
+  膀胱刺激症状（化学性膀胱炎）：最常见。
 表现：尿频、尿急、尿痛、排尿时有烧灼感，或下腹部/膀胱区不适、坠胀感。
 原因：药物对膀胱黏膜的化学刺激。
 特点：通常发生在灌注后几小时内，持续1-3天逐渐缓解。
@@ -4376,7 +4353,7 @@
 2.严重全身不适，如剧烈寒战。
 3.肉芽肿性前列腺炎或附睾炎。
 4.BCG全身感染（播散性BCG感染）：极其罕见但非常严重，可导致肺炎、肝炎、骨髓炎等，表现为持续高热、咳嗽、黄疸、骨痛等。
-二、灌注期间及灌注后的重要注意事项
+ 二、灌注期间及灌注后的重要注意事项
 为了最大程度发挥疗效并减少副作用，请严格遵守以下医嘱和注意事项：
 灌注前准备：
 1.排空膀胱：治疗前尽量排空小便，以利于药物在膀胱内充分停留。
@@ -4385,20 +4362,20 @@
 1.变换体位：灌注后，医生会要求您在躺椅上每15-30分钟变换一次体位（如左侧卧、平躺、右侧卧、俯卧）。这是为了让药物与膀胱各个壁充分接触，尤其是顶壁。
 2.严格保留药物：药物需在膀胱内保留 1-2小时（具体时间遵医嘱）。这是治疗起效的必要时间，请尽量忍耐。
 3.排尿注意：
-到时间后，第一次排尿务必在马桶内进行。因为排出的尿液中含有药物，需避免溅到皮肤或眼睛。女性患者应坐下排尿，以防飞溅。
-排尿后，应立即用大量清水冲洗马桶，并彻底洗手和会阴部。
-建议在治疗后6小时内，每次排尿都采取上述防护措施。
-生活与自我管理注意事项：
+  到时间后，第一次排尿务必在马桶内进行。因为排出的尿液中含有药物，需避免溅到皮肤或眼睛。女性患者应坐下排尿，以防飞溅。
+  排尿后，应立即用大量清水冲洗马桶，并彻底洗手和会阴部。
+  建议在治疗后6小时内，每次排尿都采取上述防护措施。
+ 生活与自我管理注意事项：
 1.大量饮水，但“错时”进行：
-灌注后的 头1-2小时（药物保留期间）不要饮水，以免稀释药物或过早产生尿意。
-完成首次排尿后，应开始大量饮水（每天至少2升），以促进药物代谢、稀释尿液、减轻刺激症状。
+  灌注后的 头1-2小时（药物保留期间）不要饮水，以免稀释药物或过早产生尿意。
+  完成首次排尿后，应开始大量饮水（每天至少2升），以促进药物代谢、稀释尿液、减轻刺激症状。
 2.观察并记录症状：记录排尿感受、体温、有无血尿等，复诊时告知医生。
 3.区分正常反应与危险信号：
-正常/可耐受：轻度尿频尿急、轻微血尿、低热（&lt;38.5℃）且一天内自行消退、轻度乏力。
-需联系医生：剧烈膀胱疼痛无法忍受、持续高热（&gt;38.5℃）、严重血尿（有大量血块）、寒战、全身皮疹、关节剧痛、呼吸困难等。出现这些症状，应立即就医。
+  正常/可耐受：轻度尿频尿急、轻微血尿、低热（&lt;38.5℃）且一天内自行消退、轻度乏力。
+  需联系医生：剧烈膀胱疼痛无法忍受、持续高热（&gt;38.5℃）、严重血尿（有大量血块）、寒战、全身皮疹、关节剧痛、呼吸困难等。出现这些症状，应立即就医。
 4.性生活和避孕：
-治疗期间及治疗后一周内，建议使用安全套，因为药物可能通过精液或阴道分泌物影响伴侣。
-BCG灌注期间，禁止无保护的性生活。
+  治疗期间及治疗后一周内，建议使用安全套，因为药物可能通过精液或阴道分泌物影响伴侣。
+  BCG灌注期间，禁止无保护的性生活。
 5.坚持完成疗程：灌注治疗是一个完整的计划（如：每周1次，连续6周的诱导治疗，之后是长达1-3年的维持治疗）。不要因为暂时的副作用而自行中断，应与医生沟通调整方案，而非放弃。
 6.与医生充分沟通：治疗前告知医生您的所有健康状况（如活动性结核、免疫缺陷、尿路感染等，尤其是BCG治疗的禁忌症）。治疗中及时反馈副作用，医生可以通过调整药物剂量、给药速度、或使用对症药物（如止痛药、解热药）来帮助您更好地耐受。
 总结
@@ -4439,8 +4416,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌术后灌注治疗有什么副作用？要注意什么？
-"膀胱癌术后膀胱灌注治疗的副作用主要集中在泌尿系统局部，全身副作用较少见，具体副作用和注意事项如下：
+          <t>膀胱癌术后膀胱灌注治疗的副作用主要集中在泌尿系统局部，全身副作用较少见，具体副作用和注意事项如下：
 一、 常见副作用
 膀胱刺激症状
 这是最常见的局部反应，表现为 尿频、尿急、尿痛，部分患者还会出现下腹部坠胀、隐痛。
@@ -4470,7 +4446,7 @@
 注意个人卫生：保持外阴清洁，预防尿路感染。
 其他重要提醒
 严格遵医嘱规律灌注：灌注治疗的疗程（如每周 1 次 ×8 周，每月 1 次 ×10 个月）是根据复发风险制定的，不可擅自中断，否则会大幅降低预防复发的效果。
-定期复查：灌注期间仍需按计划做膀胱镜、尿常规等检查，评估疗效和膀胱黏膜情况"</t>
+定期复查：灌注期间仍需按计划做膀胱镜、尿常规等检查，评估疗效和膀胱黏膜情况</t>
         </is>
       </c>
     </row>
@@ -4507,8 +4483,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌术后灌注治疗有什么副作用？要注意什么？
-常见的副作用包括：
+          <t>常见的副作用包括：
 膀胱刺激症状：这是最常见的副作用，表现为尿频、尿急、尿痛、排尿困难和耻骨上区疼痛。这些症状通常在灌注后数小时至数天内出现，程度轻重不一。
 血尿：部分患者在灌注后可能出现镜下血尿或肉眼血尿，一般较轻微，可自行缓解。
 发热：少数患者可能出现低热，通常不需要特殊处理，可自行消退。
@@ -4563,42 +4538,41 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>7.70多岁老人膀胱癌适合手术吗？
-这是一个非常关键且常见的问题。答案是：70多岁的老人患膀胱癌，完全有接受手术的可能，但“是否适合”不取决于年龄本身，而取决于一个全面的、个体化的评估。
+          <t>这是一个非常关键且常见的问题。答案是：70多岁的老人患膀胱癌，完全有接受手术的可能，但“是否适合”不取决于年龄本身，而取决于一个全面的、个体化的评估。
 简单地说，年龄不是手术的绝对禁区，但需要更审慎的评估。 现代医学更关注的是 “生理年龄”而非“实际年龄” ，即老人的整体身体状况、器官功能以及肿瘤的具体情况。
 以下是决定手术与否的核心评估维度和决策思路：
 一、手术决策的金字塔：三大评估维度
 决定是否手术、做什么手术，医生主要从以下三个方面综合考量：
 1.肿瘤情况（这是决定治疗目标的根本）
-分期与分级：
-非肌层浸润性膀胱癌（NMIBC）：这类肿瘤通常采用 经尿道膀胱肿瘤电切术（TURBT）。这是一种微创手术，通过尿道进入，没有体表切口，创伤小、恢复快。对于绝大多数能耐受麻醉的70多岁老人，TURBT通常是首选且安全有效的治疗方式。 后续可能需要进行膀胱灌注治疗。
-肌层浸润性膀胱癌（MIBC）或高风险NMIBC：这时需要考虑 根治性膀胱切除术（切除整个膀胱+周围淋巴结，男性可能包括前列腺，女性可能包括子宫附件）。这是一个大手术，决策需格外谨慎。
+ 分期与分级：
+  非肌层浸润性膀胱癌（NMIBC）：这类肿瘤通常采用 经尿道膀胱肿瘤电切术（TURBT）。这是一种微创手术，通过尿道进入，没有体表切口，创伤小、恢复快。对于绝大多数能耐受麻醉的70多岁老人，TURBT通常是首选且安全有效的治疗方式。 后续可能需要进行膀胱灌注治疗。
+  肌层浸润性膀胱癌（MIBC）或高风险NMIBC：这时需要考虑 根治性膀胱切除术（切除整个膀胱+周围淋巴结，男性可能包括前列腺，女性可能包括子宫附件）。这是一个大手术，决策需格外谨慎。
 2.患者的全身状况与器官功能（这是评估手术风险的核心）
 医生会进行一系列评估：
-心肺功能：心脏是否能承受麻醉和手术？肺功能如何？常需做心电图、心脏超声、肺功能测试。
-肾功能：手术（尤其是根治术）对肾脏有影响，术前肾功能必须达标。
-营养状况：有无贫血、低蛋白血症？营养良好的老人恢复更快。
-合并症：是否患有高血压、糖尿病、冠心病、慢性肺病等？这些疾病控制得是否稳定？
-日常生活能力：老人能否自理、散步、上下楼？这是评估其生理储备和康复潜力的直观指标。
-认知与精神状况：能否理解并配合治疗？
+  心肺功能：心脏是否能承受麻醉和手术？肺功能如何？常需做心电图、心脏超声、肺功能测试。
+  肾功能：手术（尤其是根治术）对肾脏有影响，术前肾功能必须达标。
+  营养状况：有无贫血、低蛋白血症？营养良好的老人恢复更快。
+  合并症：是否患有高血压、糖尿病、冠心病、慢性肺病等？这些疾病控制得是否稳定？
+  日常生活能力：老人能否自理、散步、上下楼？这是评估其生理储备和康复潜力的直观指标。
+  认知与精神状况：能否理解并配合治疗？
 3.患者及家属的意愿与支持系统
-治疗目标：是追求根治，还是以控制症状、提高生活质量为主？
-对风险的接受度：能否接受大手术可能带来的并发症风险？
-家庭支持：术后需要家人精心的护理和支持，家庭照护能力非常重要。
+  治疗目标：是追求根治，还是以控制症状、提高生活质量为主？
+  对风险的接受度：能否接受大手术可能带来的并发症风险？
+  家庭支持：术后需要家人精心的护理和支持，家庭照护能力非常重要。
 二、如果无法进行根治性大手术，有哪些替代方案？
 对于身体状况不适合或不愿接受根治性膀胱切除术的高龄患者，仍有多种有效选择：
 1.保留膀胱的综合治疗：
-最大限度的TURBT：尽可能彻底地切除可见肿瘤。
-联合放化疗：对于肌层浸润性癌，这是一种成熟的保留膀胱方案，疗效与根治术相当，但对身体条件有一定要求。
+  最大限度的TURBT：尽可能彻底地切除可见肿瘤。
+  联合放化疗：对于肌层浸润性癌，这是一种成熟的保留膀胱方案，疗效与根治术相当，但对身体条件有一定要求。
 2.微创/姑息性手术：
-对于引起出血、梗阻等症状的肿瘤，可以进行 姑息性TURBT，以减轻症状、提高生活质量为目标。
+  对于引起出血、梗阻等症状的肿瘤，可以进行 姑息性TURBT，以减轻症状、提高生活质量为目标。
 3.药物治疗：
-全身治疗：如果肿瘤已转移或风险极高，可采用免疫治疗、靶向治疗或化疗（需评估肾功能和全身状况）。
+  全身治疗：如果肿瘤已转移或风险极高，可采用免疫治疗、靶向治疗或化疗（需评估肾功能和全身状况）。
 膀胱灌注治疗：主要用于TURBT术后预防复发。
 给患者家属的行动建议：
 1.寻求多学科团队（MDT）诊疗：这是最重要的第一步。应前往有能力开展MDT的医院（通常是三甲医院泌尿外科），由泌尿外科医生、肿瘤内科医生、放疗科医生、麻醉科医生、影像科医生等共同会诊，为老人制定最个性化的方案。
@@ -4643,8 +4617,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>7.70多岁老人膀胱癌适合手术吗？
-"70 多岁老人患膀胱癌是否适合手术，没有绝对的答案，核心取决于 肿瘤分期分级、老人的身体基础状况、合并症情况 这三大关键因素，需要医生综合评估后决定。
+          <t>70 多岁老人患膀胱癌是否适合手术，没有绝对的答案，核心取决于 肿瘤分期分级、老人的身体基础状况、合并症情况 这三大关键因素，需要医生综合评估后决定。
 1. 肿瘤的分期和分级是首要判断依据
 非肌层浸润性膀胱癌（Ta、T1 期）
 这类肿瘤局限在膀胱黏膜层或黏膜下层，推荐的手术方式是经尿道膀胱肿瘤电切术（TURBT）。
@@ -4666,7 +4639,7 @@
 对于晚期患者，以支持治疗为主，缓解血尿、尿频等症状，提高生活质量。
 总结
 70 多岁老人并非手术的绝对禁忌人群，微创手术（如 TURBT）对多数身体状况尚可的老人是可行的；但根治性大手术则需要严格权衡利弊。
-最终方案一定要由泌尿外科、麻醉科医生共同评估，结合老人的肿瘤情况和身体耐受度来确定，同时也要尊重老人和家属的意愿。"</t>
+最终方案一定要由泌尿外科、麻醉科医生共同评估，结合老人的肿瘤情况和身体耐受度来确定，同时也要尊重老人和家属的意愿。</t>
         </is>
       </c>
     </row>
@@ -4703,8 +4676,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>70多岁老人膀胱癌适合手术吗？
-对70多岁的患者，是否能手术取决于肿瘤的分期/分级、全身耐受性与预期寿命的综合评估。年龄不是绝对禁忌，临床上不少高龄患者在充分评估后成功接受了手术；例如有89岁患者完成膀胱全切的报道。相反，若合并严重心、肺、脑等基础病且控制不佳，手术风险会明显升高，需要慎重权衡。
+          <t>对70多岁的患者，是否能手术取决于肿瘤的分期/分级、全身耐受性与预期寿命的综合评估。年龄不是绝对禁忌，临床上不少高龄患者在充分评估后成功接受了手术；例如有89岁患者完成膀胱全切的报道。相反，若合并严重心、肺、脑等基础病且控制不佳，手术风险会明显升高，需要慎重权衡。
 常见手术方式与适用情形
 经尿道膀胱肿瘤切除术（TURBT）：适用于非肌层浸润性膀胱癌（NMIBC），创伤小、恢复快，是多数早期患者的首选。术后通常需规范的膀胱内灌注化疗/免疫治疗以降低复发风险。
 根治性膀胱切除术（RC）±尿流改道：适用于肌层浸润性膀胱癌（MIBC）或高危NMIBC，需在评估可耐受的前提下进行。
@@ -4751,13 +4723,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>8.70多岁膀胱癌怎么治疗方案？
-对于70多岁的膀胱癌患者，治疗方案必须个体化制定，需要综合权衡三大核心因素：1. 肿瘤的具体情况（分期、分级、类型）；2. 患者的全身身体状况（器官功能、体能状态）；3. 患者及家属的治疗意愿和生活质量期望。
+          <t>对于70多岁的膀胱癌患者，治疗方案必须个体化制定，需要综合权衡三大核心因素：1. 肿瘤的具体情况（分期、分级、类型）；2. 患者的全身身体状况（器官功能、体能状态）；3. 患者及家属的治疗意愿和生活质量期望。
 年龄本身不是决定治疗方案的唯一标准，但高龄往往意味着可能需要更精细地平衡疗效与风险。
 以下是基于不同情况的分析和治疗思路框架，最终方案务必由泌尿外科、肿瘤内科、放疗科等多学科团队与患者及家属共同商讨决定。
 第一步：明确诊断与全面评估（这是所有决策的基础）
@@ -4765,7 +4736,7 @@
 2.  患者身体状况评估：重要脏器功能：心、肺、肝、肾功能是否能耐受手术、麻醉或化疗。体能状态评分：常用ECOG评分（04分），01分通常表示体力较好，能耐受积极治疗；2分以上则需更谨慎。合并症：是否有严重的心脑血管疾病、糖尿病、慢性阻塞性肺病等。
 第二步：根据分期和身体状况制定治疗方案
 情况一：非肌层浸润性膀胱癌（早期）目标：保留膀胱，预防复发和进展。首选治疗：经尿道膀胱肿瘤电切术。这是微创手术，通过尿道切除肿瘤，对身体打击小，非常适合高龄患者。
-术后灌注治疗（降低复发风险）：低危患者：术后单次即刻灌注化疗。 中高危患者：需进行规律灌注（化疗药或卡介苗）。卡介苗灌注效果最好，但可能引起发热、膀胱刺激等副作用，需评估患者耐受性。如果无法耐受，可选用化疗药物灌注。 密切随访：定期膀胱镜复查是关键。
+ 术后灌注治疗（降低复发风险）：低危患者：术后单次即刻灌注化疗。 中高危患者：需进行规律灌注（化疗药或卡介苗）。卡介苗灌注效果最好，但可能引起发热、膀胱刺激等副作用，需评估患者耐受性。如果无法耐受，可选用化疗药物灌注。 密切随访：定期膀胱镜复查是关键。
 情况二：肌层浸润性膀胱癌（核心决策点）
 这是治疗的关键和难点，有以下几种路径：路径A：根治性治疗（追求治愈）—— 适用于身体状况良好（ECOG 01分）的患者1.  标准方案：新辅助化疗 + 根治性膀胱切除术。这是最有可能治愈的方案。挑战：需评估患者对以顺铂为基础的化疗的耐受性（对肾功能、听力、体力要求高）。如果肾功能不佳，可考虑改用卡铂或吉西他滨单药等替代方案。 手术方式：可选择开放手术或腹腔镜/机器人辅助微创手术（创伤小、恢复快，对高龄者可能更有优势）。 尿流改道：与患者充分沟通。 回肠膀胱术：需腹壁造口佩戴造口袋，手术相对简单，并发症少。 原位新膀胱术：生活质量高，但手术更复杂、耗时更长，对患者肾功能、肠道功能、学习排尿能力要求高，需严格筛选。
 2.  保膀胱综合治疗： 方案：最大限度电切术 + 同步放化疗。 适用：适用于肿瘤较小、单发、无肾积水，且患者强烈希望保留膀胱，或因合并症无法耐受大手术，但能耐受放疗者。优势：避免了膀胱切除和尿流改道。 风险：严格的终身随访，仍有复发和进展风险，失败后需行“补救性膀胱切除”。
@@ -4815,8 +4786,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>8.70多岁膀胱癌怎么治疗方案
-"70 多岁膀胱癌患者的治疗方案，核心是兼顾肿瘤控制与老人身体耐受度，优先选择创伤小、风险低的方案，具体需结合肿瘤分期分级和老人身体基础状况综合制定，以下是分情况的治疗建议：
+          <t>70 多岁膀胱癌患者的治疗方案，核心是兼顾肿瘤控制与老人身体耐受度，优先选择创伤小、风险低的方案，具体需结合肿瘤分期分级和老人身体基础状况综合制定，以下是分情况的治疗建议：
 一、 非肌层浸润性膀胱癌（Ta、T1 期，肿瘤局限黏膜 / 黏膜下层）
 这是老年人最常见的类型，治疗以微创 + 局部灌注为主，尽量避免大手术：
 首选手术：经尿道膀胱肿瘤电切术（TURBT）
@@ -4842,7 +4812,7 @@
 关键注意事项
 必须多学科评估：泌尿外科、麻醉科、肿瘤科医生共同评估老人的手术耐受度、基础病控制情况，制定个性化方案。
 优先保障生活质量：老年人治疗的核心不是 “彻底消灭肿瘤”，而是在控制症状的前提下，避免治疗带来的严重痛苦。
-密切随访：无论选择哪种方案，都需要定期复查（超声、尿常规、肿瘤标志物等），及时调整治疗策略。"</t>
+密切随访：无论选择哪种方案，都需要定期复查（超声、尿常规、肿瘤标志物等），及时调整治疗策略。</t>
         </is>
       </c>
     </row>
@@ -4879,29 +4849,28 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>70多岁膀胱癌怎么治疗方案？
-一、先做分期与全身评估
-• 明确分期与分级：以经尿道膀胱肿瘤切除（TURBT）获取病理，判断是否为非肌层浸润性（NMIBC）或肌层浸润性（MIBC），这是选择治疗路径的基石。
-• 评估可耐受性：高龄并非手术禁忌，但需综合心肺功能、肝肾功能、营养状态及合并症控制情况，必要时行多学科会诊（MDT）与围手术期优化。
-• 明确治疗目标：在根治与生活质量之间权衡，尤其关注术后尿流改道方式对日常起居的影响。
+          <t>一、先做分期与全身评估
+明确分期与分级：以经尿道膀胱肿瘤切除（TURBT）获取病理，判断是否为非肌层浸润性（NMIBC）或肌层浸润性（MIBC），这是选择治疗路径的基石。  
+评估可耐受性：高龄并非手术禁忌，但需综合心肺功能、肝肾功能、营养状态及合并症控制情况，必要时行多学科会诊（MDT）与围手术期优化。  
+明确治疗目标：在根治与生活质量之间权衡，尤其关注术后尿流改道方式对日常起居的影响。 
 二、按分期选择治疗方案
 分期/情形 首选方案 可选/补充 关键注意点
 NMIBC（非肌层浸润） TURBT 完整切除 术后膀胱内灌注：化疗（如丝裂霉素C、表柔比星等）或BCG；少数局限且反复复发者考虑膀胱部分切除 灌注可降低复发风险；高龄患者需关注灌注相关刺激症状与耐受性
 MIBC（肌层浸润）且可耐受手术 根治性膀胱切除+尿流改道（男性常需一并处理前列腺/精囊） 围手术期/术后系统治疗（化疗/免疫治疗）视体能决定 根治术创伤大，需充分评估与围手术期管理
 MIBC但不耐受大手术 放疗（可联合化疗）或系统治疗 必要时行姑息性手术（如造瘘）以缓解血尿/梗阻 以症状控制与生活质量为主
 晚期/转移性 系统治疗：含铂类联合化疗（如吉西他滨+顺铂）或免疫治疗 放疗用于缓解骨痛、出血等；姑息性手术改善排尿/出血 高龄对化疗耐受性较差，需严密监测不良反应并加强支持治疗
-以上路径强调“分期先行、个体化选择”，高龄患者同样可在评估后获得根治机会或获得良好的症状控制。
+以上路径强调“分期先行、个体化选择”，高龄患者同样可在评估后获得根治机会或获得良好的症状控制。 
 三、70+患者的特殊考虑
-• 手术可行性：70岁可以手术，前提是身体可耐受且检查达标；若合并多种基础病或术前评估不过关，宜采取非手术或姑息策略。
-• 围手术期管理：重视心肺功能、肝肾功能、营养优化与并发症预防，必要时MDT制定个体化方案。
-• 治疗目标：在延长生存与生活质量之间平衡，尤其重视术后尿流改道对日常活动的影响与护理便利性。
+手术可行性：70岁可以手术，前提是身体可耐受且检查达标；若合并多种基础病或术前评估不过关，宜采取非手术或姑息策略。  
+围手术期管理：重视心肺功能、肝肾功能、营养优化与并发症预防，必要时MDT制定个体化方案。  
+治疗目标：在延长生存与生活质量之间平衡，尤其重视术后尿流改道对日常活动的影响与护理便利性。 
 四、治疗后的随访与生活质量
-• 随访要点：按分期与风险分层进行膀胱镜复查、影像学评估与尿细胞学等，早期发现问题、及时处理。
-• 支持治疗：贯穿全程的疼痛管理、营养支持、心理干预，有助于提升体力与生活质量。
-• 生活方式：戒烟、充足饮水、规律作息与适度运动，按医嘱完成灌注或系统治疗，减少并发症与复发风险。
+随访要点：按分期与风险分层进行膀胱镜复查、影像学评估与尿细胞学等，早期发现问题、及时处理。  
+支持治疗：贯穿全程的疼痛管理、营养支持、心理干预，有助于提升体力与生活质量。  
+生活方式：戒烟、充足饮水、规律作息与适度运动，按医嘱完成灌注或系统治疗，减少并发症与复发风险。 
 五、就医与下一步建议
-• 尽快就诊泌尿外科，完善膀胱镜+病理、影像与实验室检查，明确分期/分级与可切除性。
-• 与医生重点讨论：是否手术、术式与尿流改道选择、是否需要系统治疗及其强度、术后随访节奏与生活质量目标。</t>
+尽快就诊泌尿外科，完善膀胱镜+病理、影像与实验室检查，明确分期/分级与可切除性。  
+与医生重点讨论：是否手术、术式与尿流改道选择、是否需要系统治疗及其强度、术后随访节奏与生活质量目标。</t>
         </is>
       </c>
     </row>
@@ -4933,27 +4902,26 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>10.膀胱癌有哪些靶向药？
-膀胱癌的靶向治疗药物相对有限，目前主要针对晚期或转移性尿路上皮癌（膀胱癌最常见的类型）。靶向药通常用于特定基因突变或特定情况的患者，且必须在肿瘤科医生指导下，根据基因检测结果和病情阶段决定使用。
+          <t>膀胱癌的靶向治疗药物相对有限，目前主要针对晚期或转移性尿路上皮癌（膀胱癌最常见的类型）。靶向药通常用于特定基因突变或特定情况的患者，且必须在肿瘤科医生指导下，根据基因检测结果和病情阶段决定使用。
 以下是目前已获批准或临床上常用的膀胱癌靶向药物：
-1. 靶向FGFR的抑制剂
-厄达替尼（Erdafitinib）适用患者：用于治疗局部晚期或转移性尿路上皮癌，且肿瘤具有FGFR2或FGFR3基因突变的患者（需经过基因检测确认）。作用机制：抑制成纤维细胞生长因子受体（FGFR），阻断促进肿瘤生长的信号通路。备注：这是首个针对膀胱癌FGFR突变的靶向药，适用于含铂化疗失败后的患者。
+ 1. 靶向FGFR的抑制剂
+   厄达替尼（Erdafitinib）适用患者：用于治疗局部晚期或转移性尿路上皮癌，且肿瘤具有FGFR2或FGFR3基因突变的患者（需经过基因检测确认）。作用机制：抑制成纤维细胞生长因子受体（FGFR），阻断促进肿瘤生长的信号通路。备注：这是首个针对膀胱癌FGFR突变的靶向药，适用于含铂化疗失败后的患者。
 2. 抗体药物偶联物（ADCs，兼具靶向和化疗作用）
-恩诺单抗（Enfortumab vedotin）适用患者：用于治疗局部晚期或转移性尿路上皮癌，且既往接受过含铂化疗和免疫治疗（PD1/PDL1抑制剂） 后病情进展的患者。作用机制：靶向细胞表面的Nectin4蛋白，携带化疗药物直接进入癌细胞。
-戈沙妥珠单抗（Sacituzumab govitecan适用患者：用于治疗局部晚期或转移性尿路上皮癌，且既往接受过含铂化疗和免疫治疗的患者。作用机制：靶向Trop2蛋白，携带拓扑异构酶抑制剂至癌细胞。
+   恩诺单抗（Enfortumab vedotin）适用患者：用于治疗局部晚期或转移性尿路上皮癌，且既往接受过含铂化疗和免疫治疗（PD1/PDL1抑制剂） 后病情进展的患者。作用机制：靶向细胞表面的Nectin4蛋白，携带化疗药物直接进入癌细胞。
+   戈沙妥珠单抗（Sacituzumab govitecan适用患者：用于治疗局部晚期或转移性尿路上皮癌，且既往接受过含铂化疗和免疫治疗的患者。作用机制：靶向Trop2蛋白，携带拓扑异构酶抑制剂至癌细胞。
 3. 抗血管生成靶向药（多靶点抑制剂）
-舒尼替尼（Sunitinib）、索凡替尼（Surufatinib）等适用患者：这些药物并非膀胱癌一线治疗，但在临床研究中尝试用于晚期患者的后续治疗，通常联合化疗或免疫治疗。作用机制：抑制肿瘤血管生成（如VEGFR靶点），切断肿瘤营养供应。
+   舒尼替尼（Sunitinib）、索凡替尼（Surufatinib）等适用患者：这些药物并非膀胱癌一线治疗，但在临床研究中尝试用于晚期患者的后续治疗，通常联合化疗或免疫治疗。作用机制：抑制肿瘤血管生成（如VEGFR靶点），切断肿瘤营养供应。
 重要补充说明
 1. 靶向药使用前提：
-大多数靶向药需通过基因检测（如FGFR突变、HER2扩增等）或生物标志物检测筛选适用人群。
-通常用于晚期转移性膀胱癌，且在传统治疗（如手术、化疗、免疫治疗）失败后。
+   大多数靶向药需通过基因检测（如FGFR突变、HER2扩增等）或生物标志物检测筛选适用人群。
+   通常用于晚期转移性膀胱癌，且在传统治疗（如手术、化疗、免疫治疗）失败后。
 2. 联合治疗趋势：
-目前临床研究更多探索靶向药与免疫治疗（如PD1/PDL1抑制剂）或化疗的联合应用，以提高疗效。
+   目前临床研究更多探索靶向药与免疫治疗（如PD1/PDL1抑制剂）或化疗的联合应用，以提高疗效。
 3. 其他潜在靶点药物：
 HER2抑制剂（如曲妥珠单抗）：仅用于少数HER2阳性的膀胱癌患者，尚非常规应用。
 PARP抑制剂（如奥拉帕利）：在具有DNA修复基因突变（如BRCA）的患者中研究，但尚未成为标准治疗。
@@ -5001,8 +4969,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>10.膀胱癌有哪些靶向药？
-"膀胱癌的靶向治疗药物主要针对特定的分子靶点，多用于晚期或转移性膀胱癌患者，尤其是化疗失败后的二线及以上治疗。目前获批或临床常用的靶向药主要分为以下几类：
+          <t>膀胱癌的靶向治疗药物主要针对特定的分子靶点，多用于晚期或转移性膀胱癌患者，尤其是化疗失败后的二线及以上治疗。目前获批或临床常用的靶向药主要分为以下几类：
 1. 抗血管生成靶向药
 这类药物通过抑制肿瘤新生血管的形成，切断肿瘤的营养供应，从而抑制肿瘤生长和转移，是膀胱癌靶向治疗的主要方向。
 厄达替尼（Erdafitinib）
@@ -5028,7 +4995,7 @@
 重要注意事项
 靶向治疗需做基因检测：靶向药的使用前提是患者肿瘤组织中存在对应的靶点（如 FGFR 突变、HER2 过表达），因此治疗前需要进行基因检测或免疫组化，明确靶点后再选择药物。
 适用人群有限：目前膀胱癌靶向药主要用于晚期、转移性或化疗失败的患者，早中期膀胱癌仍以手术和灌注治疗为主。
-存在副作用：靶向药也可能有副作用，如厄达替尼可能导致口腔溃疡、高磷血症；ADC 药物可能引起骨髓抑制、周围神经病变等，需在医生指导下使用并监测不良反应。"</t>
+存在副作用：靶向药也可能有副作用，如厄达替尼可能导致口腔溃疡、高磷血症；ADC 药物可能引起骨髓抑制、周围神经病变等，需在医生指导下使用并监测不良反应。</t>
         </is>
       </c>
     </row>
@@ -5065,26 +5032,25 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌有哪些靶向药？
-一、已证实疗效且临床常用的靶向药
-• FGFR 抑制剂：厄达替尼（Erdafitinib）
-• 适用人群：携带FGFR2/FGFR3突变或融合的局部晚期或转移性尿路上皮癌成人患者。
-• 使用要点：用药前需进行FGFR 基因检测；常见不良反应包括口腔炎、疲劳、肌酐升高等，需监测肾功能与口腔状况。
-• 定位：目前最具明确分子选择性的膀胱癌靶向药之一。
+          <t>一、已证实疗效且临床常用的靶向药
+FGFR 抑制剂：厄达替尼（Erdafitinib）  
+适用人群：携带FGFR2/FGFR3突变或融合的局部晚期或转移性尿路上皮癌成人患者。  
+使用要点：用药前需进行FGFR 基因检测；常见不良反应包括口腔炎、疲劳、肌酐升高等，需监测肾功能与口腔状况。  
+定位：目前最具明确分子选择性的膀胱癌靶向药之一。 
 二、证据有限或主要处于研究阶段的靶向药
-• EGFR 通路抑制剂：如吉非替尼、厄洛替尼、西妥昔单抗、拉帕替尼等。
-• VEGFR 通路抑制剂：如舒尼替尼、索拉非尼、帕唑帕尼、凡德他尼、贝伐珠单抗。
-• FGFR 其他抑制剂：如多韦替尼（Dovitinib）。
-• mTOR 抑制剂：如依维莫司。
-• 说明：上述药物在膀胱癌中的疗效证据有限，多为II期或回顾性研究，尚未成为标准治疗；部分药物仅在特定情境或临床试验中考虑使用，需由医生评估后决定。
+EGFR 通路抑制剂：如吉非替尼、厄洛替尼、西妥昔单抗、拉帕替尼等。  
+VEGFR 通路抑制剂：如舒尼替尼、索拉非尼、帕唑帕尼、凡德他尼、贝伐珠单抗。  
+FGFR 其他抑制剂：如多韦替尼（Dovitinib）。  
+mTOR 抑制剂：如依维莫司。  
+说明：上述药物在膀胱癌中的疗效证据有限，多为II期或回顾性研究，尚未成为标准治疗；部分药物仅在特定情境或临床试验中考虑使用，需由医生评估后决定。 
 三、与靶向易混淆的常用药物（非靶向）
-• 免疫治疗（检查点抑制剂）：如帕博利珠单抗、阿替利珠单抗等，属于免疫药物而非靶向药，但在局部晚期或转移性膀胱癌治疗中具有重要作用。
-• 化疗药物：如顺铂、吉西他滨等，常用于晚期或辅助/新辅助治疗，亦非靶向药。
+免疫治疗（检查点抑制剂）：如帕博利珠单抗、阿替利珠单抗等，属于免疫药物而非靶向药，但在局部晚期或转移性膀胱癌治疗中具有重要作用。  
+化疗药物：如顺铂、吉西他滨等，常用于晚期或辅助/新辅助治疗，亦非靶向药。 
 四、用药选择与检测建议
-• 明确病理类型与分期：靶向治疗目前主要用于晚期/转移性尿路上皮癌，早期患者以手术及膀胱内灌注（如BCG/化疗）为主。
-• 进行分子检测：拟考虑厄达替尼时，优先检测FGFR2/FGFR3突变或融合。
-• 治疗路径：靶向药在多数情况下用于后线或特定指征；是否联合化疗/免疫治疗由MDT个体化决策。
-• 不良反应管理：关注口腔炎、疲劳、肾功能变化（FGFR 抑制剂）及高血压、手足综合征、出血风险（多靶点TKI）等，按医嘱监测与处理。
+明确病理类型与分期：靶向治疗目前主要用于晚期/转移性尿路上皮癌，早期患者以手术及膀胱内灌注（如BCG/化疗）为主。  
+进行分子检测：拟考虑厄达替尼时，优先检测FGFR2/FGFR3突变或融合。  
+治疗路径：靶向药在多数情况下用于后线或特定指征；是否联合化疗/免疫治疗由MDT个体化决策。  
+不良反应管理：关注口腔炎、疲劳、肾功能变化（FGFR 抑制剂）及高血压、手足综合征、出血风险（多靶点TKI）等，按医嘱监测与处理。 
 医疗提示：本内容为健康科普，不能替代医生面诊与处方。涉及具体用药与基因检测，请在泌尿外科/肿瘤科医生指导下进行，切勿自行购药或更换方案。</t>
         </is>
       </c>
@@ -5117,34 +5083,33 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>11.卡介苗能治疗膀胱癌吗？
-这是一个非常重要且常见的问题。答案是：能，但仅限于特定类型和分期的膀胱癌，而不是所有膀胱癌。
+          <t>这是一个非常重要且常见的问题。答案是：能，但仅限于特定类型和分期的膀胱癌，而不是所有膀胱癌。
 卡介苗（Bacillus CalmetteGuérin, BCG）是预防结核病的疫苗，但它在非肌层浸润性膀胱癌（NMIBC）的治疗中扮演着极其重要的角色，被认为是其一线免疫治疗药物。
 下面为您详细解释：
 1. 适用情况：非肌层浸润性膀胱癌
-什么是NMIBC：指癌细胞仅局限于膀胱黏膜层或黏膜下层，未侵犯到膀胱肌肉层。这是大约75%新发膀胱癌患者的初始诊断类型。
-高危NMIBC：尤其是原位癌（CIS）、高级别Ta期和T1期肿瘤，术后复发和进展风险很高。卡介苗正是这些高危患者的标准治疗方案。
+   什么是NMIBC：指癌细胞仅局限于膀胱黏膜层或黏膜下层，未侵犯到膀胱肌肉层。这是大约75%新发膀胱癌患者的初始诊断类型。
+   高危NMIBC：尤其是原位癌（CIS）、高级别Ta期和T1期肿瘤，术后复发和进展风险很高。卡介苗正是这些高危患者的标准治疗方案。
 2. 治疗目的：预防复发和阻止进展
-主要目标：不是直接杀死已形成的肿瘤（手术已切除），而是通过激发局部免疫反应，清除残余的、肉眼看不见的癌细胞，并预防新肿瘤的形成。
-效果：对于高危患者，单纯手术切除后复发率可高达60%90%。使用卡介苗灌注后，可以将复发率降低约50%70%，并能显著降低肿瘤向肌层浸润性膀胱癌进展的风险。
+   主要目标：不是直接杀死已形成的肿瘤（手术已切除），而是通过激发局部免疫反应，清除残余的、肉眼看不见的癌细胞，并预防新肿瘤的形成。
+   效果：对于高危患者，单纯手术切除后复发率可高达60%90%。使用卡介苗灌注后，可以将复发率降低约50%70%，并能显著降低肿瘤向肌层浸润性膀胱癌进展的风险。
 3. 如何使用：膀胱灌注
-过程：通过导尿管，将卡介苗（一种活的、减毒的牛型结核分枝杆菌）溶液直接灌入膀胱。
-周期：通常为诱导治疗（术后开始，每周一次，连续6周），然后进行维持治疗（在后续的3、6、12、18、24个月等时间点，再进行一系列灌注），总疗程通常为13年。研究表明，维持治疗对长期疗效至关重要。
+   过程：通过导尿管，将卡介苗（一种活的、减毒的牛型结核分枝杆菌）溶液直接灌入膀胱。
+   周期：通常为诱导治疗（术后开始，每周一次，连续6周），然后进行维持治疗（在后续的3、6、12、18、24个月等时间点，再进行一系列灌注），总疗程通常为13年。研究表明，维持治疗对长期疗效至关重要。
 4. 作用原理（为什么能抗癌？）
-卡介苗进入膀胱后，会吸引并激活人体自身的免疫细胞（如巨噬细胞、T淋巴细胞等） 聚集到膀胱壁。这些被强烈激活的免疫细胞不仅攻击卡介苗菌，还会“误伤”或识别并攻击具有相似表面抗原的膀胱癌细胞，从而产生强大的局部抗癌免疫效应。
+   卡介苗进入膀胱后，会吸引并激活人体自身的免疫细胞（如巨噬细胞、T淋巴细胞等） 聚集到膀胱壁。这些被强烈激活的免疫细胞不仅攻击卡介苗菌，还会“误伤”或识别并攻击具有相似表面抗原的膀胱癌细胞，从而产生强大的局部抗癌免疫效应。
 5. 不适用的情况
-肌层浸润性膀胱癌：癌细胞已侵犯膀胱肌肉层。此时，主要的治疗方法是根治性膀胱切除术、化疗、放疗或联合治疗。卡介苗对此类癌症无效。
-某些特殊情况：患者有活动性结核感染、严重免疫功能低下、或膀胱因手术/放疗有大面积损伤时，禁用卡介苗。
-对卡介苗无反应或复发：部分患者使用卡介苗后效果不佳或肿瘤复发，此时需要更换治疗方案，如使用吉西他滨等化疗药物进行膀胱灌注，或考虑根治性手术。
+   肌层浸润性膀胱癌：癌细胞已侵犯膀胱肌肉层。此时，主要的治疗方法是根治性膀胱切除术、化疗、放疗或联合治疗。卡介苗对此类癌症无效。
+   某些特殊情况：患者有活动性结核感染、严重免疫功能低下、或膀胱因手术/放疗有大面积损伤时，禁用卡介苗。
+   对卡介苗无反应或复发：部分患者使用卡介苗后效果不佳或肿瘤复发，此时需要更换治疗方案，如使用吉西他滨等化疗药物进行膀胱灌注，或考虑根治性手术。
 6. 可能的副作用
-卡介苗灌注是一种强烈的免疫刺激，副作用较为常见，但大多轻微且可管理：
-常见：膀胱刺激症状（尿频、尿急、排尿疼痛）、血尿、流感样症状（低热、乏力）。
-严重但罕见：持续高烧、严重全身感染（如BCG败血症）、前列腺炎、肝炎等。一旦出现高烧不退等症状，需立即就医，并使用抗结核药物治疗。
+   卡介苗灌注是一种强烈的免疫刺激，副作用较为常见，但大多轻微且可管理：
+   常见：膀胱刺激症状（尿频、尿急、排尿疼痛）、血尿、流感样症状（低热、乏力）。
+   严重但罕见：持续高烧、严重全身感染（如BCG败血症）、前列腺炎、肝炎等。一旦出现高烧不退等症状，需立即就医，并使用抗结核药物治疗。
 总结
 能治疗：卡介苗是高危非肌层浸润性膀胱癌术后预防复发和进展的“金标准”疗法。
 不能治疗：它不适用于已侵犯肌肉层的肌层浸润性膀胱癌，也不适用于所有膀胱癌患者。
@@ -5186,8 +5151,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>卡介苗能治疗膀胱癌吗？
-"卡介苗（BCG）可以用于治疗膀胱癌，且是目前浅表性膀胱癌术后辅助治疗的核心方案之一，其作用机制和临床应用具有明确的循证医学证据支撑。
+          <t>卡介苗（BCG）可以用于治疗膀胱癌，且是目前浅表性膀胱癌术后辅助治疗的核心方案之一，其作用机制和临床应用具有明确的循证医学证据支撑。
 一、 适用范围与核心作用
 卡介苗治疗膀胱癌的适用场景并非晚期转移性膀胱癌，而是针对非肌层浸润性膀胱癌（NMIBC），具体包括：
 经尿道膀胱肿瘤电切术（TURBT）后，用于降低肿瘤复发风险、延缓疾病进展；
@@ -5209,7 +5173,7 @@
 五、 局限性
 对肌层浸润性膀胱癌或转移性膀胱癌无效；
 存在一定比例的耐药病例，约 10%~30% 的患者对卡介苗治疗无反应或治疗后复发；
-治疗周期长，患者依从性对疗效影响较大"</t>
+治疗周期长，患者依从性对疗效影响较大</t>
         </is>
       </c>
     </row>
@@ -5246,32 +5210,31 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>卡介苗能治疗膀胱癌吗？
-卡介苗（BCG）是治疗膀胱癌的重要手段，但不是所有类型的膀胱癌都适用。
+          <t>卡介苗（BCG）是治疗膀胱癌的重要手段，但不是所有类型的膀胱癌都适用。
 具体来说：
 1.  卡介苗的主要作用：
-◦   预防复发：对于非肌层浸润性膀胱癌（NMIBC），特别是高危NMIBC（如高级别Ta、T1期肿瘤，或伴有原位癌CIS），经尿道膀胱肿瘤切除（TURBT）后，膀胱内灌注卡介苗是目前最有效的预防复发的方法之一。
-◦   延缓进展：卡介苗还能在一定程度上延缓肿瘤向肌层浸润性膀胱癌（MIBC）进展的风险。
+    ◦   预防复发：对于非肌层浸润性膀胱癌（NMIBC），特别是高危NMIBC（如高级别Ta、T1期肿瘤，或伴有原位癌CIS），经尿道膀胱肿瘤切除（TURBT）后，膀胱内灌注卡介苗是目前最有效的预防复发的方法之一。
+    ◦   延缓进展：卡介苗还能在一定程度上延缓肿瘤向肌层浸润性膀胱癌（MIBC）进展的风险。
 2.  卡介苗适用的膀胱癌类型：
-◦   主要适用于非肌层浸润性膀胱癌（NMIBC），尤其是那些复发风险较高的患者。
-◦   对于原位癌（CIS），卡介苗是标准的治疗选择。
+    ◦   主要适用于非肌层浸润性膀胱癌（NMIBC），尤其是那些复发风险较高的患者。
+    ◦   对于原位癌（CIS），卡介苗是标准的治疗选择。
 3.  卡介苗的作用机制：
-◦   卡介苗是一种减毒的牛型结核杆菌，将其注入膀胱后，会刺激膀胱黏膜产生强烈的免疫反应，从而激活机体的免疫系统来攻击和清除残留的癌细胞，达到治疗和预防复发的目的。
+    ◦   卡介苗是一种减毒的牛型结核杆菌，将其注入膀胱后，会刺激膀胱黏膜产生强烈的免疫反应，从而激活机体的免疫系统来攻击和清除残留的癌细胞，达到治疗和预防复发的目的。
 4.  卡介苗的使用方法：
-◦   通常在TURBT术后2周左右开始进行膀胱内灌注。
-◦   初始诱导阶段通常需要每周灌注一次，连续6周。
-◦   之后可能还需要进行维持治疗，以维持长期的疗效，减少复发风险。维持治疗的方案会根据患者的具体情况而定。
+    ◦   通常在TURBT术后2周左右开始进行膀胱内灌注。
+    ◦   初始诱导阶段通常需要每周灌注一次，连续6周。
+    ◦   之后可能还需要进行维持治疗，以维持长期的疗效，减少复发风险。维持治疗的方案会根据患者的具体情况而定。
 5.  卡介苗的副作用：
-◦   膀胱刺激症状：如尿频、尿急、尿痛、排尿困难等，这是最常见的副作用。
-◦   血尿：部分患者在灌注后可能出现镜下或肉眼血尿。
-◦   发热：少数患者可能出现低热。
-◦   过敏反应：极少数患者可能出现皮疹、瘙痒等过敏反应。
-◦   更严重的并发症：如膀胱挛缩、前列腺炎、附睾炎等，但发生率较低。
+    ◦   膀胱刺激症状：如尿频、尿急、尿痛、排尿困难等，这是最常见的副作用。
+    ◦   血尿：部分患者在灌注后可能出现镜下或肉眼血尿。
+    ◦   发热：少数患者可能出现低热。
+    ◦   过敏反应：极少数患者可能出现皮疹、瘙痒等过敏反应。
+    ◦   更严重的并发症：如膀胱挛缩、前列腺炎、附睾炎等，但发生率较低。
 6.  卡介苗的禁忌症：
-◦   对卡介苗或其成分过敏者。
-◦   存在活动性结核病或其他严重感染的患者。
-◦   严重的免疫功能低下者。
-◦   急性膀胱炎、膀胱穿孔等情况。
+    ◦   对卡介苗或其成分过敏者。
+    ◦   存在活动性结核病或其他严重感染的患者。
+    ◦   严重的免疫功能低下者。
+    ◦   急性膀胱炎、膀胱穿孔等情况。
 总结来说：
 卡介苗是治疗非肌层浸润性膀胱癌（NMIBC），特别是高危NMIBC和原位癌（CIS）的一种有效方法，主要用于预防复发和延缓进展。但它并非适用于所有类型的膀胱癌，其使用需要在医生的指导下进行，并密切关注可能出现的副作用。如果你或你认识的人患有膀胱癌，请务必咨询专业的泌尿外科医生，他们会根据具体情况制定最合适的治疗方案。</t>
         </is>
@@ -5305,13 +5268,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>13.浸润性膀胱癌必须做膀胱全切手术吗？有没有保守治疗方案？
-这是一个非常关键且实际的问题，答案是：不一定必须立即全切，但“根治性膀胱全切术”是目前治疗肌层浸润性膀胱癌的“金标准”和最主要的治愈性手段。 确实存在一些旨在保留膀胱的“保守治疗方案”，但这些方案有严格的适用条件和自身的风险，需要在经验丰富的医疗团队指导下进行权衡选择。下面我为您详细梳理两种路径的核心要点：
+          <t>这是一个非常关键且实际的问题，答案是：不一定必须立即全切，但“根治性膀胱全切术”是目前治疗肌层浸润性膀胱癌的“金标准”和最主要的治愈性手段。 确实存在一些旨在保留膀胱的“保守治疗方案”，但这些方案有严格的适用条件和自身的风险，需要在经验丰富的医疗团队指导下进行权衡选择。下面我为您详细梳理两种路径的核心要点：
 路径一：标准治疗方案 —— 根治性膀胱全切术：这是最经典、研究最充分、长期生存率最高的方法。为什么它是“金标准”？  1. 根治性：目的是完整切除膀胱及周围的潜在转移区域（通常包括男性前列腺、精囊，女性子宫、部分阴道前壁）以及盆腔淋巴结，力求“根治”。2. 防复发：能最大程度去除局部病灶，防止肿瘤在膀胱内复发或侵犯周围器官。3. 长期数据支持：对于符合条件的患者，其提供的长期无病生存率和总生存率是目前所有治疗方案中最高的。
 术后生活质量问题（尿流改道）： 回肠膀胱术：最常用。取一段小肠作为输出道，在腹壁造口，需要终身佩戴造口袋收集尿液。原位新膀胱术：取一段肠道重塑成一个新“膀胱”，与尿道吻合，患者术后可经尿道自主排尿，生活质量较高。这是目前最理想的保功能术式，但对患者年龄、体力、肾功能、肿瘤位置（尿道需安全）及手术技巧要求高。其他方式：如可控性尿囊等。
 路径二：保膀胱综合治疗方案（三联疗法）这是一种“化疗+放疗+最大限度经尿道膀胱肿瘤电切术” 的组合方案。其目标是在不切除膀胱的情况下，达到与根治性手术相似的长期生存效果。适用人群（严格筛选）：1.  肿瘤为单发、相对较小。2.  没有肾积水（说明输尿管口未受侵）。3. 肿瘤未侵犯到膀胱颈或尿道。 4.  首次经尿道电切能达到肉眼完全切除（达到T0状态）。 5. 患者年龄较大、身体状况无法耐受大手术，或个人强烈拒绝膀胱切除。
@@ -5357,8 +5319,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>浸润性膀胱癌必须做膀胱全切手术吗？有没有保守治疗方案？
-肌层浸润性膀胱癌（MIBC）并非必须行膀胱全切手术，治疗方案需根据肿瘤分期、患者身体状况、意愿等综合判断，存在保留膀胱的综合保守治疗方案，但需严格把握适应证。
+          <t>肌层浸润性膀胱癌（MIBC）并非必须行膀胱全切手术，治疗方案需根据肿瘤分期、患者身体状况、意愿等综合判断，存在保留膀胱的综合保守治疗方案，但需严格把握适应证。
 一、 核心治疗方案分类及适用场景
 1. 膀胱全切手术（金标准方案）
 这是肌层浸润性膀胱癌的首选根治性方案，尤其适用于以下情况：
@@ -5377,6 +5338,21 @@
 同步放化疗：这是保留膀胱方案的关键。放疗靶区覆盖膀胱及盆腔淋巴结，同时联合化疗药物（如顺铂），利用放化疗的协同作用杀灭残留肿瘤细胞，降低复发风险；
 术后随访与再评估：治疗后需定期行膀胱镜、影像学检查，若肿瘤复发，需及时转为膀胱全切手术。
 二、 两种方案的疗效对比
+治疗方案
+5 年生存率
+膀胱保留率
+复发风险
+生活质量影响
+膀胱全切术
+50%~70%
+0
+较低（局部复发率＜10%）
+尿流改道可能影响生活便利性
+保留膀胱综合治疗
+40%~60%
+60%~70%
+较高（约 30%~40% 患者需二次全切）
+保留膀胱功能，生活质量相对更高
 三、 保守治疗的局限性
 严格适应证限制：仅适用于早期肌层浸润病例，T3/T4 期肿瘤不建议采用；
 复发率高：约 1/3 的患者会在 2~3 年内复发，复发后多数需接受膀胱全切；
@@ -5418,28 +5394,27 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>浸润性膀胱癌必须做膀胱全切手术吗？有没有保守治疗方案？
-是否必须行膀胱全切
-并非所有肌层浸润性膀胱癌（MIBC）都必须行根治性膀胱全切（RC）。RC联合盆腔淋巴结清扫长期被视为标准治疗，原因在于单纯经尿道膀胱肿瘤电切（TURBT）难以彻底清除浸润病灶，存在进展与转移风险；但当患者不适合大手术或强烈希望保留膀胱时，在严格选择的前提下，可采用保留膀胱的综合治疗方案。需要强调的是，保留膀胱并不等于“少治疗”，通常意味着更严密的全身治疗与随访。
+          <t>是否必须行膀胱全切
+并非所有肌层浸润性膀胱癌（MIBC）都必须行根治性膀胱全切（RC）。RC联合盆腔淋巴结清扫长期被视为标准治疗，原因在于单纯经尿道膀胱肿瘤电切（TURBT）难以彻底清除浸润病灶，存在进展与转移风险；但当患者不适合大手术或强烈希望保留膀胱时，在严格选择的前提下，可采用保留膀胱的综合治疗方案。需要强调的是，保留膀胱并不等于“少治疗”，通常意味着更严密的全身治疗与随访。 
 可考虑保留膀胱的情形
-• 肿瘤局限、单发且位于可切除区域，患者强烈希望保留膀胱并能配合综合治疗与随访。
-• 全身状况良好，能够耐受化疗/放疗；关键器官功能（心、肺、肾等）可满足治疗需求。
-• 接受“先治疗、再评估”的策略：先行TURBT联合系统/放疗，达临床完全缓解（cCR）后继续严密监测；一旦出现复发，及时转为RC。
-• 所在中心具备成熟的多学科团队（MDT）与放疗能力，能提供规范化实施与质量控制。
+肿瘤局限、单发且位于可切除区域，患者强烈希望保留膀胱并能配合综合治疗与随访。  
+全身状况良好，能够耐受化疗/放疗；关键器官功能（心、肺、肾等）可满足治疗需求。  
+接受“先治疗、再评估”的策略：先行TURBT联合系统/放疗，达临床完全缓解（cCR）后继续严密监测；一旦出现复发，及时转为RC。  
+所在中心具备成熟的多学科团队（MDT）与放疗能力，能提供规范化实施与质量控制。 
 可选的保守治疗方案
-• 三模态保膀胱（TMT）：最大化安全切除的TURBT + 同步放化疗（以顺铂为主），随后按疗效决定巩固治疗或转RC。多项长期研究显示，选择得当的患者可获得与RC相近的生存，同时保留功能性膀胱；对诱导后未达cCR者，推荐挽救性RC。
-• TURBT + 系统治疗（化疗/免疫）保膀胱：例如吉西他滨+顺铂（GC）+ 纳武利尤单抗（Opdivo）诱导，达到cCR后继续免疫维持并密切随访；未达cCR或复发则转RC。该策略在近年研究中可使多数MIBC患者避免即刻全切。
-• 膀胱部分切除术：适用于肿瘤较小、位置局限（如侧后壁/顶部）且切缘可达阴性的患者；术后通常需配合化疗/放疗以降低复发风险。
-• 放疗作为保膀胱方案的基石：现代以同步放化疗为主；单纯放疗目前主要用于不能耐受化疗者，历史上单用放疗的疗效已明显被联合方案取代。
+三模态保膀胱（TMT）：最大化安全切除的TURBT + 同步放化疗（以顺铂为主），随后按疗效决定巩固治疗或转RC。多项长期研究显示，选择得当的患者可获得与RC相近的生存，同时保留功能性膀胱；对诱导后未达cCR者，推荐挽救性RC。   
+TURBT + 系统治疗（化疗/免疫）保膀胱：例如吉西他滨+顺铂（GC）+ 纳武利尤单抗（Opdivo）诱导，达到cCR后继续免疫维持并密切随访；未达cCR或复发则转RC。该策略在近年研究中可使多数MIBC患者避免即刻全切。   
+膀胱部分切除术：适用于肿瘤较小、位置局限（如侧后壁/顶部）且切缘可达阴性的患者；术后通常需配合化疗/放疗以降低复发风险。   
+放疗作为保膀胱方案的基石：现代以同步放化疗为主；单纯放疗目前主要用于不能耐受化疗者，历史上单用放疗的疗效已明显被联合方案取代。 
 保膀胱策略的疗效与风险要点
-• 疗效数据：在选定人群中，TMT的5年总体生存（OS）约60%–72%，5年膀胱保留率约60%；部分中心长期随访显示≥80%的生存者仍保留功能膀胱。
-• 复发与挽救：保膀胱并非避免复发，而是“先控瘤、后严密监测”；一旦局部复发，标准做法是及时行挽救性RC，总体仍可取得良好结局。
-• 毒性与依从性：同步放化疗的≥3级胃肠/泌尿毒性约1%–5%；需有经验的团队进行毒副反应管理与支持治疗，患者需具备良好依从性与随访条件。
+疗效数据：在选定人群中，TMT的5年总体生存（OS）约60%–72%，5年膀胱保留率约60%；部分中心长期随访显示≥80%的生存者仍保留功能膀胱。   
+复发与挽救：保膀胱并非避免复发，而是“先控瘤、后严密监测”；一旦局部复发，标准做法是及时行挽救性RC，总体仍可取得良好结局。   
+毒性与依从性：同步放化疗的≥3级胃肠/泌尿毒性约1%–5%；需有经验的团队进行毒副反应管理与支持治疗，患者需具备良好依从性与随访条件。 
 就医与决策建议
-• 尽快完成TURBT取病理+分期（含影像与必要活检），明确是否真性MIBC及是否有淋巴结/远处转移。
-• 与泌尿外科、肿瘤内科、放疗科进行MDT讨论，评估手术可切除性与保膀胱可行性，并制定“诱导—评估—巩固/转治”路径。
-• 如拟保膀胱，确保可在有经验的中心实施同步放化疗或系统治疗，并签署严密随访与“复发即转RC”的预案。
-• 医疗提示：以上为健康科普，不能替代个体化诊疗；具体方案需由医生结合病理分期、全身状况与中心能力综合判定。</t>
+尽快完成TURBT取病理+分期（含影像与必要活检），明确是否真性MIBC及是否有淋巴结/远处转移。  
+与泌尿外科、肿瘤内科、放疗科进行MDT讨论，评估手术可切除性与保膀胱可行性，并制定“诱导—评估—巩固/转治”路径。  
+如拟保膀胱，确保可在有经验的中心实施同步放化疗或系统治疗，并签署严密随访与“复发即转RC”的预案。  
+医疗提示：以上为健康科普，不能替代个体化诊疗；具体方案需由医生结合病理分期、全身状况与中心能力综合判定。</t>
         </is>
       </c>
     </row>
@@ -5471,33 +5446,32 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>3.膀胱癌患者有哪些饮食禁忌？
-这是一个非常实际且重要的问题。对于膀胱癌患者而言，虽然没有一个绝对的、适用于所有人的“禁忌食谱”，但科学的饮食管理对降低复发风险、促进身体恢复、提高治疗效果和生活质量至关重要。
+          <t>这是一个非常实际且重要的问题。对于膀胱癌患者而言，虽然没有一个绝对的、适用于所有人的“禁忌食谱”，但科学的饮食管理对降低复发风险、促进身体恢复、提高治疗效果和生活质量至关重要。
 总体原则是：均衡营养，增强免疫力；避免明确有害的物质；保持健康的体重。
 以下是具体的饮食建议和注意事项：
 一、强烈建议避免或严格限制的（“禁忌”核心）
 1.  吸烟与酒精：
-吸烟：是膀胱癌最明确的危险因素之一。烟草中的致癌物经尿液排出，长期直接刺激膀胱黏膜。确诊后必须立即彻底戒烟，这是最重要的“饮食禁忌”（吸烟虽非饮食，但密切相关）。
+ 吸烟：是膀胱癌最明确的危险因素之一。烟草中的致癌物经尿液排出，长期直接刺激膀胱黏膜。确诊后必须立即彻底戒烟，这是最重要的“饮食禁忌”（吸烟虽非饮食，但密切相关）。
 酒精：酒精代谢可能对膀胱有刺激，且可能干扰身体代谢和免疫功能。建议尽量避免或严格限量，特别是在治疗期间。
 2.某些可能有害的食物与饮品：
-含砷饮用水：长期饮用高砷水是风险因素。确保饮用水安全。
-大量摄入加工肉类和红肉：一些研究提示，大量食用腌制、熏制、加工的肉类（如火腿、香肠、培根）可能与风险增加有关。建议减少食用频率和分量，选择新鲜禽肉、鱼肉作为蛋白质来源。
-过度摄入脂肪和油炸食物：高脂饮食可能促进炎症，不利于整体健康。
-某些传统“发物”：如民间所说的狗肉、羊肉等，从现代医学看，并无直接证据表明会加速膀胱癌生长，但因其可能属于高脂或不易消化蛋白质，在治疗期间若身体不适，可适当减少。
+  含砷饮用水：长期饮用高砷水是风险因素。确保饮用水安全。
+  大量摄入加工肉类和红肉：一些研究提示，大量食用腌制、熏制、加工的肉类（如火腿、香肠、培根）可能与风险增加有关。建议减少食用频率和分量，选择新鲜禽肉、鱼肉作为蛋白质来源。
+  过度摄入脂肪和油炸食物：高脂饮食可能促进炎症，不利于整体健康。
+  某些传统“发物”：如民间所说的狗肉、羊肉等，从现代医学看，并无直接证据表明会加速膀胱癌生长，但因其可能属于高脂或不易消化蛋白质，在治疗期间若身体不适，可适当减少。
 二、需谨慎对待或根据治疗阶段调整的
 1.饮水习惯：
-禁忌：饮水不足！ 这是大忌。充足饮水（每天1.5-2升以上）可以稀释尿液中的致癌物，减少对膀胱的刺激，是预防复发的重要措施。但如有肾功能问题，需遵医嘱。
-注意：治疗期间（如膀胱灌注后、放疗期间），医生可能会对饮水量和饮水时间有特殊要求，请遵医嘱。
+  禁忌：饮水不足！ 这是大忌。充足饮水（每天1.5-2升以上）可以稀释尿液中的致癌物，减少对膀胱的刺激，是预防复发的重要措施。但如有肾功能问题，需遵医嘱。
+  注意：治疗期间（如膀胱灌注后、放疗期间），医生可能会对饮水量和饮水时间有特殊要求，请遵医嘱。
 2.刺激性与调味品：
-对于正在进行治疗（尤其是放疗、灌注化疗）或伴有膀胱刺激症状（尿频、尿急、尿痛）的患者，过辣、过酸、过甜的食物及浓茶、咖啡可能会加重膀胱刺激症状。建议观察个人反应，如有不适，则应减少或避免。
+  对于正在进行治疗（尤其是放疗、灌注化疗）或伴有膀胱刺激症状（尿频、尿急、尿痛）的患者，过辣、过酸、过甜的食物及浓茶、咖啡可能会加重膀胱刺激症状。建议观察个人反应，如有不适，则应减少或避免。
 3.保健品与补品：
-禁忌：盲目进补！ 某些补品或高剂量维生素/矿物质补充剂可能干扰化疗或放疗效果。
-关键建议：在服用任何维生素（特别是大剂量维生素C、E、硒等）、中药或保健品前，务必咨询您的主治医生或临床营养师，切勿自行服用。
+  禁忌：盲目进补！ 某些补品或高剂量维生素/矿物质补充剂可能干扰化疗或放疗效果。
+  关键建议：在服用任何维生素（特别是大剂量维生素C、E、硒等）、中药或保健品前，务必咨询您的主治医生或临床营养师，切勿自行服用。
 三、积极鼓励摄入的（构建健康饮食模式）
 1.丰富的蔬菜和水果：
 尤其是富含抗氧化剂和植物化学物的种类，如 十字花科蔬菜（西兰花、菜花、卷心菜）、番茄（富含番茄红素）、绿叶蔬菜、浆果类（蓝莓、草莓）和柑橘类水果。它们有助于对抗氧化损伤，增强免疫力。
@@ -5508,9 +5482,9 @@
 4.健康的饮水：
 白开水是最佳选择。可以适量饮用清淡的绿茶（富含儿茶素），但避免过浓。
 根据治疗阶段的特别提醒：
-手术（膀胱切除术）后：初期饮食需从流质、半流质逐步过渡，少食多餐，避免腹胀。长期来看，根治性膀胱切除+尿流改道术后，需注意预防尿液酸中毒，可能需要多食碱性食物（如蔬菜水果），并遵医嘱定期监测。
-化疗/放疗期间：可能伴有恶心、呕吐、食欲不振、味觉改变。此时饮食目标是 “保证营养摄入” ，应选择清淡、易消化、高蛋白的食物，少食多餐。可尝试改变食物性状（如做成糊、羹）。必要时使用营养补充剂，并咨询临床营养师。
-膀胱灌注期间：灌注当天可适当减少饮水以避免尿频不适，但其他时间仍需保证充足饮水。
+   手术（膀胱切除术）后：初期饮食需从流质、半流质逐步过渡，少食多餐，避免腹胀。长期来看，根治性膀胱切除+尿流改道术后，需注意预防尿液酸中毒，可能需要多食碱性食物（如蔬菜水果），并遵医嘱定期监测。
+   化疗/放疗期间：可能伴有恶心、呕吐、食欲不振、味觉改变。此时饮食目标是 “保证营养摄入” ，应选择清淡、易消化、高蛋白的食物，少食多餐。可尝试改变食物性状（如做成糊、羹）。必要时使用营养补充剂，并咨询临床营养师。
+   膀胱灌注期间：灌注当天可适当减少饮水以避免尿频不适，但其他时间仍需保证充足饮水。
 总结与行动建议：
 1.戒烟限酒，保证饮水：这是两条铁的纪律。
 2.遵循“彩虹饮食”原则：让您的餐盘色彩丰富，多吃不同颜色的蔬菜水果。
@@ -5554,8 +5528,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>3.膀胱癌患者有哪些饮食禁忌？
-"膀胱癌患者的饮食管理核心是减轻膀胱负担、降低肿瘤复发风险、增强身体抵抗力，以下是需要注意的饮食禁忌和相关建议：
+          <t>膀胱癌患者的饮食管理核心是减轻膀胱负担、降低肿瘤复发风险、增强身体抵抗力，以下是需要注意的饮食禁忌和相关建议：
 一、 明确需要避免的食物
 辛辣刺激性食物
 辣椒、花椒、生姜、大蒜、芥末等，这类食物会刺激膀胱黏膜，加重尿频、尿急等不适症状，尤其对于术后或化疗期间的患者，黏膜本身较为脆弱，更要严格避免。
@@ -5574,7 +5547,7 @@
 多吃鸡蛋、牛奶、鱼肉、豆制品等优质蛋白，帮助修复身体组织，增强免疫力；搭配新鲜蔬菜和水果，补充维生素和膳食纤维。
 规律饮食，少食多餐
 尤其对于化疗、放疗期间的患者，胃肠道功能较弱，少食多餐可以减轻肠胃负担，避免腹胀、恶心等不适。
-需要注意的是，饮食禁忌是辅助康复的手段，不能替代正规的治疗和随访，具体饮食方案还可以根据患者的治疗阶段、身体状况，咨询主治医生或临床营养师。"</t>
+需要注意的是，饮食禁忌是辅助康复的手段，不能替代正规的治疗和随访，具体饮食方案还可以根据患者的治疗阶段、身体状况，咨询主治医生或临床营养师。</t>
         </is>
       </c>
     </row>
@@ -5611,8 +5584,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌患者有哪些饮食禁忌？
-膀胱癌患者的饮食管理主要是为了避免刺激膀胱、减少复发风险、保证营养摄入以支持治疗和康复。以下是一些常见的饮食注意事项和禁忌：
+          <t>膀胱癌患者的饮食管理主要是为了避免刺激膀胱、减少复发风险、保证营养摄入以支持治疗和康复。以下是一些常见的饮食注意事项和禁忌：
 避免辛辣刺激食物：如辣椒、花椒、生姜、大蒜（生）、芥末等，这些食物可能刺激膀胱黏膜，加重尿路刺激症状。
 限制酒精和咖啡因摄入：酒精和咖啡因（咖啡、浓茶、可乐、巧克力等）具有利尿作用，可能增加膀胱负担，并可能刺激膀胱黏膜。
 减少高脂肪、高胆固醇食物：如油炸食品、动物内脏、肥肉等。这类食物可能影响身体的代谢和免疫功能。
@@ -5662,20 +5634,19 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>16.男性膀胱癌患者术后，对夫妻生活、生育有影响吗？
-这是一个非常重要且实际的问题。膀胱癌手术对男性患者的性功能和生育能力确实可能产生显著影响，但其程度主要取决于手术的范围和类型。简单来说：非肌层浸润性膀胱癌的手术（经尿道电切术）通常影响很小；而肌层浸润性膀胱癌的标准手术（根治性膀胱切除术）则影响很大。
+          <t>这是一个非常重要且实际的问题。膀胱癌手术对男性患者的性功能和生育能力确实可能产生显著影响，但其程度主要取决于手术的范围和类型。简单来说：非肌层浸润性膀胱癌的手术（经尿道电切术）通常影响很小；而肌层浸润性膀胱癌的标准手术（根治性膀胱切除术）则影响很大。
 以下是详细的分情况说明：
-一、非肌层浸润性膀胱癌（电切术后）：手术方式：经尿道膀胱肿瘤电切术
+ 一、非肌层浸润性膀胱癌（电切术后）：手术方式：经尿道膀胱肿瘤电切术
 对夫妻生活的影响：通常很小或没有直接影响。该手术通过尿道进行，不涉及前列腺、精囊和支配阴茎勃起的神经。患者恢复后，性功能一般能保持术前水平。
 对生育的影响：理论上没有直接影响。因为手术不涉及睾丸、输精管等生殖器官。但需注意两点：
-1.  如果术后需要进行膀胱灌注化疗或卡介苗治疗，在治疗期间，药物可能对精子的质量和活力产生暂时性影响。建议在积极治疗期间采取避孕措施，并在治疗结束后咨询医生关于精子质量的恢复情况。
-2.  极少数情况下，如果肿瘤位于膀胱颈或前列腺尿道部，电切手术可能损伤膀胱颈的闭合功能，导致逆行射精（精液射入膀胱而非经尿道排出），这会影响自然受孕，但通常可以通过辅助生殖技术解决。
-二、肌层浸润性膀胱癌（根治性膀胱切除术后）
+    1.  如果术后需要进行膀胱灌注化疗或卡介苗治疗，在治疗期间，药物可能对精子的质量和活力产生暂时性影响。建议在积极治疗期间采取避孕措施，并在治疗结束后咨询医生关于精子质量的恢复情况。
+    2.  极少数情况下，如果肿瘤位于膀胱颈或前列腺尿道部，电切手术可能损伤膀胱颈的闭合功能，导致逆行射精（精液射入膀胱而非经尿道排出），这会影响自然受孕，但通常可以通过辅助生殖技术解决。
+ 二、肌层浸润性膀胱癌（根治性膀胱切除术后）
 这是影响最大的情况。手术切除范围包括：整个膀胱、前列腺、精囊，以及盆腔淋巴结。
 1. 对夫妻生活（性功能）的影响
 根治性手术不可避免地会损伤控制阴茎勃起的盆腔自主神经丛，导致术后出现不同程度的勃起功能障碍。
@@ -5690,15 +5661,15 @@
 时机：在确诊后，手术或化疗开始前，尽快联系生殖医学中心。
 流程：进行精子质量检查，并冷冻保存足够数量的精子。
 意义：为术后通过辅助生殖技术（如试管婴儿） 拥有自己的生物学后代保留了唯一的机会。这是根治术前必须考虑的“生育力保存”措施。
-三、尿流改道方式对生活的影响
+ 三、尿流改道方式对生活的影响
 术后排尿方式的改变也会间接影响夫妻生活和自信心。
 回肠膀胱术（腹壁造口）：需终身佩戴造口袋。这可能对患者的身体形象和性生活自信造成心理影响。但通过正确护理和使用专用器具，完全可以进行正常的性生活。
 原位新膀胱术：从腹部看不出异常，可经尿道自主排尿。在身体形象和性生活心理层面更具优势。
-总结与核心建议
+ 总结与核心建议
 1.  明确手术类型：首先确认是电切术还是根治术，这是判断影响程度的基础。
 2.  根治术前必须沟通：
-性功能保留：与主刀医生深入探讨实施 “保留神经的手术” 的可行性和预期效果。
-生育力保存：如果未来有生育可能，务必在术前进行精子冷冻！
+    性功能保留：与主刀医生深入探讨实施 “保留神经的手术” 的可行性和预期效果。
+    生育力保存：如果未来有生育可能，务必在术前进行精子冷冻！
 3.  术后积极寻求帮助：如果出现性功能障碍，应主动向泌尿外科或男科医生求助，现代医学有多种有效的方法可以帮助改善。
 4.  夫妻沟通至关重要：手术后，双方需要时间适应身体和心理的变化。开放、坦诚的沟通，互相理解和支持，是维持亲密关系最重要的基础。必要时可寻求心理咨询师的帮助。
 请务必与您的医疗团队（特别是主刀医生）在手术前就这些问题进行充分、详细的沟通，让他们了解您的关切，以便共同制定最适合您的个体化治疗方案。</t>
@@ -5738,8 +5709,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌患者术后，对夫妻生活、生育有影响吗？
-男性膀胱癌患者术后对夫妻生活和生育的影响，取决于手术方式和治疗方案，不同术式的影响程度差异较大，具体如下：
+          <t>男性膀胱癌患者术后对夫妻生活和生育的影响，取决于手术方式和治疗方案，不同术式的影响程度差异较大，具体如下：
 一、 对夫妻生活的影响
 1. 经尿道膀胱肿瘤电切术（TURBT）—— 影响较小
 这是浅表性膀胱癌的首选术式，属于微创手术，不损伤膀胱外的生殖系统和盆底神经。
@@ -5804,30 +5774,29 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌患者术后，对夫妻生活、生育有影响吗？
-一、对夫妻生活的影响
+          <t>一、对夫妻生活的影响
 1.  保留膀胱的手术（如TURBT、膀胱部分切除）：
-◦   这类手术通常对性功能影响较小。TURBT（经尿道膀胱肿瘤电切术）主要是切除膀胱内的肿瘤，不涉及生殖器官，因此对勃起功能和射精功能基本没有影响。
-◦   膀胱部分切除术如果切除范围不大，且没有损伤到支配阴茎勃起的神经血管束，对性生活的影响也相对较小。但手术本身可能会给患者带来一定的心理压力，从而影响性欲和性生活质量。
+    ◦   这类手术通常对性功能影响较小。TURBT（经尿道膀胱肿瘤电切术）主要是切除膀胱内的肿瘤，不涉及生殖器官，因此对勃起功能和射精功能基本没有影响。
+    ◦   膀胱部分切除术如果切除范围不大，且没有损伤到支配阴茎勃起的神经血管束，对性生活的影响也相对较小。但手术本身可能会给患者带来一定的心理压力，从而影响性欲和性生活质量。
 2.  根治性膀胱切除术（RC）：
-◦   这是影响最大的一种手术方式。由于手术需要切除膀胱、前列腺、精囊腺，有时还会切除部分尿道，因此会对男性的性功能产生显著影响。
-◦   勃起功能障碍（ED）：手术可能会损伤支配阴茎勃起的神经血管束，导致勃起功能障碍。发生率因手术技巧、是否保留神经以及患者年龄、基础疾病等因素而异，文献报道差异较大，从20%到80%不等。
-◦   逆行射精：由于手术切除了精囊腺和输精管末端，并且膀胱颈部的结构发生改变，患者在性高潮时精液无法正常射出体外，而是逆行流入膀胱，称为逆行射精。这意味着患者仍然可以有性高潮的感觉，但无法使伴侣受孕。
-◦   性欲下降：手术创伤、术后疼痛、心理压力、激素水平变化等都可能导致性欲下降。
+    ◦   这是影响最大的一种手术方式。由于手术需要切除膀胱、前列腺、精囊腺，有时还会切除部分尿道，因此会对男性的性功能产生显著影响。
+    ◦   勃起功能障碍（ED）：手术可能会损伤支配阴茎勃起的神经血管束，导致勃起功能障碍。发生率因手术技巧、是否保留神经以及患者年龄、基础疾病等因素而异，文献报道差异较大，从20%到80%不等。
+    ◦   逆行射精：由于手术切除了精囊腺和输精管末端，并且膀胱颈部的结构发生改变，患者在性高潮时精液无法正常射出体外，而是逆行流入膀胱，称为逆行射精。这意味着患者仍然可以有性高潮的感觉，但无法使伴侣受孕。
+    ◦   性欲下降：手术创伤、术后疼痛、心理压力、激素水平变化等都可能导致性欲下降。
 二、对生育的影响
 1.  保留膀胱的手术：
-◦   如果手术没有损伤到输精管和睾丸，通常不会影响精子的生成和运输，因此对生育能力影响不大。但如果肿瘤侵犯了精囊腺或输精管，可能会对生育造成一定影响。
+    ◦   如果手术没有损伤到输精管和睾丸，通常不会影响精子的生成和运输，因此对生育能力影响不大。但如果肿瘤侵犯了精囊腺或输精管，可能会对生育造成一定影响。
 2.  根治性膀胱切除术（RC）：
-◦   由于手术切除了精囊腺和输精管末端，并且精液会逆行射入膀胱，因此患者术后基本丧失了自然生育能力。
-◦   对于有生育需求的年轻患者，可以考虑在手术前进行精子冷冻保存，以备将来使用辅助生殖技术（如试管婴儿）来实现生育愿望。
+    ◦   由于手术切除了精囊腺和输精管末端，并且精液会逆行射入膀胱，因此患者术后基本丧失了自然生育能力。
+    ◦   对于有生育需求的年轻患者，可以考虑在手术前进行精子冷冻保存，以备将来使用辅助生殖技术（如试管婴儿）来实现生育愿望。
 三、如何应对这些影响
 1.  术前沟通：在决定手术方案前，患者应与医生充分沟通，了解不同手术方式对性功能和生育能力的潜在影响，并根据自己的需求和期望做出选择。
 2.  术中保护：在进行根治性膀胱切除术时，医生会尽量采用保留神经的根治性膀胱切除术（NS-RC），以最大程度地保护患者的勃起功能。
 3.  术后康复：
-◦   心理治疗：术后出现性功能障碍和生育问题可能会给患者带来巨大的心理压力，因此需要进行心理疏导和支持，帮助患者调整心态，积极面对。
-◦   药物治疗：对于勃起功能障碍，可以在医生的指导下使用磷酸二酯酶-5抑制剂（如西地那非、他达拉非）等药物来改善勃起功能。
-◦   康复训练：进行盆底肌肉训练等康复训练，有助于改善局部的血液循环和神经功能，对性功能的恢复有一定帮助。
-◦   辅助生殖技术：对于术后丧失自然生育能力的患者，可以考虑通过人工授精或试管婴儿等辅助生殖技术来实现生育愿望。
+    ◦   心理治疗：术后出现性功能障碍和生育问题可能会给患者带来巨大的心理压力，因此需要进行心理疏导和支持，帮助患者调整心态，积极面对。
+    ◦   药物治疗：对于勃起功能障碍，可以在医生的指导下使用磷酸二酯酶-5抑制剂（如西地那非、他达拉非）等药物来改善勃起功能。
+    ◦   康复训练：进行盆底肌肉训练等康复训练，有助于改善局部的血液循环和神经功能，对性功能的恢复有一定帮助。
+    ◦   辅助生殖技术：对于术后丧失自然生育能力的患者，可以考虑通过人工授精或试管婴儿等辅助生殖技术来实现生育愿望。
 4.  夫妻沟通：患者应与伴侣坦诚沟通，共同面对术后可能出现的问题，相互理解和支持，这对于性生活的和谐和家庭的稳定非常重要。
 总结来说：男性膀胱癌患者术后对夫妻生活和生育的影响因手术方式而异。保留膀胱的手术影响较小，而根治性膀胱切除术则可能对性功能和生育能力产生显著影响。患者在术前应与医生充分沟通，了解潜在风险，并在术后积极采取应对措施，以提高生活质量。</t>
         </is>
@@ -5861,33 +5830,32 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>17.膀胱癌治疗要花多少钱？
-这是一个非常现实且重要的问题，但膀胱癌的治疗费用差异极大，无法给出一个固定数字。它就像一个“区间”，从几万到几十万甚至更高，主要取决于以下几个核心因素：
+          <t>这是一个非常现实且重要的问题，但膀胱癌的治疗费用差异极大，无法给出一个固定数字。它就像一个“区间”，从几万到几十万甚至更高，主要取决于以下几个核心因素：
 为了让您有一个更直观的理解，以下是一个基于不同治疗阶段的费用估算框架（请注意：所有费用均为大致估算，且以上海、北京等一线城市三甲医院为例，具体以医院实际结算为准，医保报销前费用）：
-一、影响费用的四大关键因素
+ 一、影响费用的四大关键因素
 1.  癌症分期与类型：非肌层浸润性膀胱癌（早期）：治疗相对简单，费用较低。肌层浸润性或晚期膀胱癌：需要综合治疗，费用呈几何级增长。
 2.  治疗方案：这是费用差异的最大来源。单纯电切手术和根治性膀胱切除术+尿流改道的费用天差地别。
 3.  治疗地区与医院：不同城市、不同医院（公立三甲 vs. 国际部/私立医院）的收费标准不同。
 4.  医保政策与自费项目： 医保报销比例：城镇职工、城乡居民医保不同，且各地报销目录和比例有差异。
-自费项目：许多靶向药、新型免疫药、部分高价耗材（如手术吻合器、造口袋）可能需完全或部分自费。
-二、各阶段治疗费用估算（人民币，医保报销前）
+  自费项目：许多靶向药、新型免疫药、部分高价耗材（如手术吻合器、造口袋）可能需完全或部分自费。
+ 二、各阶段治疗费用估算（人民币，医保报销前）
 阶段一：诊断与评估（约 0.5万  2万元）检查项目：膀胱镜+活检（约20005000元）、泌尿系增强CT/MRI（约10003000元）、全身骨扫描/ PETCT（约700012000元，后者常自费）、各项化验。 这部分费用相对固定，医保可报销大部分。
 阶段二：手术治疗（费用差异的核心）
 1.  经尿道膀胱肿瘤电切术：适合：非肌层浸润性膀胱癌。费用：约 1.5万  3万元。若肿瘤多发或较大，费用增加。后续：需加上膀胱灌注治疗的费用（化疗药或卡介苗，每月数百至数千元，持续数月到数年）。
 2.  根治性膀胱切除术 + 尿流改道术：适合：肌层浸润性膀胱癌。这是费用最高的环节。 手术及住院费用：约 820万元。 差异关键在于“尿流改道”方式：回肠膀胱术：相对标准，费用在区间下限。
 原位新膀胱术：手术更复杂，耗时更长，使用的吻合器、缝线等耗材可能更贵（部分需自费），费用接近区间上限。
-重要提示：若使用达芬奇机器人辅助手术，手术费会大幅增加（可能额外增加 3万  8万元 或更多，且大部分地区医保不报销或报销比例极低）。
+    重要提示：若使用达芬奇机器人辅助手术，手术费会大幅增加（可能额外增加 3万  8万元 或更多，且大部分地区医保不报销或报销比例极低）。
 阶段三：辅助治疗（周期长，变量大）
 1.  化疗：新辅助/辅助化疗（常用方案：GC方案吉西他滨+顺铂）。每周期费用约 0.5万  1.5万元（取决于用药和是否使用高端止吐、升白药）。通常需46个周期，总费用约 3万  9万元。大部分化疗药已入医保。
 2.  免疫治疗： 常用药物：帕博利珠单抗（K药）、替雷利珠单抗、特瑞普利单抗等。费用高昂：单次注射约 1万  3.5万元（不同药物价格不同）。重大利好：目前多个PD1抑制剂已纳入国家医保，报销后自付部分大幅降低，可能降至每月数千元。但医保有严格适应症限制（如用于术后高危辅助治疗或晚期一线联合化疗等）。
 3.  靶向治疗： 如厄达替尼（针对FGFR突变），费用极高，但已有药物通过医保谈判大幅降价并纳入医保，报销后负担减轻。抗体偶联药物（如恩诺单抗）：非常昂贵，目前大多需完全自费或参加临床试验。
 阶段四：随访与维持（长期支出）定期复查（膀胱镜、CT、化验）：每年约 0.5万1万元。造口护理用品（如适用）：每月数百至上千元。
-三、如何应对高昂费用？——实用建议
+ 三、如何应对高昂费用？——实用建议
 1.  首要依靠：国家基本医疗保险：务必参保！这是最基础的保障。了解本地医保的起付线、封顶线、报销比例和药品/项目目录。办理门诊特殊病种/慢性病备案，可以大幅提高门诊治疗（如灌注、化疗、靶向药）的报销比例。
 2.  重要补充：大病医疗保险与医疗救助：医保报销后，个人负担仍超过一定金额，可进入 “大病医保” 二次报销。对于低收入家庭，可咨询当地民政部门 “医疗救助” 政策。
 3.  商业健康保险（如有）： 如有在患病前购买的百万医疗险、重疾险，可申请理赔，有效转移经济风险。
@@ -5931,8 +5899,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌治疗要花多少钱？
-膀胱癌的治疗费用没有固定标准，主要取决于治疗方案、肿瘤分期、医院等级、地区差异以及是否使用医保报销，不同治疗路径的费用跨度极大，具体如下：
+          <t>膀胱癌的治疗费用没有固定标准，主要取决于治疗方案、肿瘤分期、医院等级、地区差异以及是否使用医保报销，不同治疗路径的费用跨度极大，具体如下：
 一、 非肌层浸润性膀胱癌（浅表性）—— 费用相对可控
 以经尿道膀胱肿瘤电切术（TURBT）+ 术后膀胱灌注治疗为核心方案，费用构成如下：
 TURBT 手术费用
@@ -5996,8 +5963,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>膀胱癌治疗要花多少钱？
-费用跨度很大，受肿瘤分期与治疗方式、医院与地区、医保报销等影响。总体上，从数万元（早期、单一治疗）到十几万—数十万元（根治术+尿流改道+综合治疗/长期维持）均可能出现。为便于预估，下面按常见项目给出典型区间与要点。
+          <t>费用跨度很大，受肿瘤分期与治疗方式、医院与地区、医保报销等影响。总体上，从数万元（早期、单一治疗）到十几万—数十万元（根治术+尿流改道+综合治疗/长期维持）均可能出现。为便于预估，下面按常见项目给出典型区间与要点。
 主要治疗项目与典型费用
 项目 典型单次/疗程费用 常见区间 说明
 经尿道膀胱肿瘤电切术（TURBT） 按次住院 1–2万元 多数非肌层浸润性病例的首选；费用随医院等级、耗材而变动
@@ -6011,21 +5977,21 @@
 检查与支持治疗 随项目 术前评估约数百–上千元；住院期间的护理/营养/并发症处理另计 复查（膀胱镜、影像）为长期支出点
 以上区间为公开渠道的典型参考，实际以就诊医院收费为准。
 影响费用的关键因素
-• 治疗方式与手术方式：TURBT费用最低；根治性膀胱切除因是否行尿流改道、腹腔镜/机器人等不同而显著波动。
-• 分期与病情复杂度：分期越晚、范围越大，手术难度与住院时长增加，费用上行。
-• 医院等级与地区差异：三甲医院与一线地区收费通常更高。
-• 耗材与药物选择：进口器械/药物价格更高；是否纳入医保决定自付比例。
-• 治疗周期与并发症：化疗/放疗周期数、是否出现感染等并发症，都会拉高总支出。
+治疗方式与手术方式：TURBT费用最低；根治性膀胱切除因是否行尿流改道、腹腔镜/机器人等不同而显著波动。  
+分期与病情复杂度：分期越晚、范围越大，手术难度与住院时长增加，费用上行。  
+医院等级与地区差异：三甲医院与一线地区收费通常更高。  
+耗材与药物选择：进口器械/药物价格更高；是否纳入医保决定自付比例。  
+治疗周期与并发症：化疗/放疗周期数、是否出现感染等并发症，都会拉高总支出。
 常见治疗路径的费用估算示例
-• 早期非肌层浸润性膀胱癌（TURBT + 术后膀胱灌注）：
-TURBT住院约1–2万元；灌注化疗约500–1000元/次，常见方案为术后每周1次×8次，随后每月1次×10次维持约1年，灌注合计约1.3–2.0万元（以吉西他滨/表柔比星等为例，部分药物可医保）。总体常见为数万元级。
-• 肌层浸润性膀胱癌行根治性膀胱切除±尿流改道：
-手术费约3–5万元；如行尿流改道，常需额外1–2万元；若选择机器人手术，整体可达≥5–8万元。术后根据病理分期与风险评估，可能追加全身化疗/放疗，总额通常进入数万—十余万元区间。
+早期非肌层浸润性膀胱癌（TURBT + 术后膀胱灌注）：  
+  TURBT住院约1–2万元；灌注化疗约500–1000元/次，常见方案为术后每周1次×8次，随后每月1次×10次维持约1年，灌注合计约1.3–2.0万元（以吉西他滨/表柔比星等为例，部分药物可医保）。总体常见为数万元级。
+肌层浸润性膀胱癌行根治性膀胱切除±尿流改道：  
+  手术费约3–5万元；如行尿流改道，常需额外1–2万元；若选择机器人手术，整体可达≥5–8万元。术后根据病理分期与风险评估，可能追加全身化疗/放疗，总额通常进入数万—十余万元区间。
 医保与减轻负担的实用建议
-• 提前向医院医保办确认：哪些药物/耗材可报销、报销比例、起付线与封顶线、异地就医结算规则。
-• 医生沟通治疗方案与替代药物（国产/进口），在保证疗效的前提下优化自付比例。
-• 关注当地医疗救助/慈善项目与医院社工服务，必要时申请经济援助。
-• 符合条件者可咨询临床试验，有机会获得免费或部分减免的药物与检查。
+提前向医院医保办确认：哪些药物/耗材可报销、报销比例、起付线与封顶线、异地就医结算规则。  
+医生沟通治疗方案与替代药物（国产/进口），在保证疗效的前提下优化自付比例。  
+关注当地医疗救助/慈善项目与医院社工服务，必要时申请经济援助。  
+符合条件者可咨询临床试验，有机会获得免费或部分减免的药物与检查。  
 以上举措可显著降低实际支出，建议在治疗前即做好费用—疗效—风险的综合权衡。</t>
         </is>
       </c>
@@ -6058,41 +6024,40 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>19.男性膀胱癌复查膀胱镜需要住院吗？
-这是一个非常实际的复查问题。简单来说，答案是：绝大多数情况下不需要住院。 膀胱镜检查是膀胱癌术后随访的常规项目，通常作为 “日间手术”或“门诊检查” 完成。
+          <t>这是一个非常实际的复查问题。简单来说，答案是：绝大多数情况下不需要住院。 膀胱镜检查是膀胱癌术后随访的常规项目，通常作为 “日间手术”或“门诊检查” 完成。
 以下是详细的说明和注意事项：
 常规复查膀胱镜：通常是门诊操作
 对于大多数情况稳定的复查患者，膀胱镜过程如下：
 1.  地点：在医院的 “日间手术中心” 或 “门诊膀胱镜检查室” 进行。
 2.  流程：
-预约：按医生嘱咐的复查时间提前预约。
-术前准备：检查前可能需要做简单的尿常规、感染筛查（如HIV、梅毒、乙肝等，这是常规手术前检查）。部分医院要求检查前禁食水几小时（尤其是如果需要麻醉的话）。
-麻醉：通常采用 “尿道表面麻醉” （将局麻药凝胶挤入尿道，等待数分钟起效）。对于疼痛敏感、焦虑或尿道狭窄的患者，可以选择 “静脉镇静麻醉” （即短时间的全麻，睡一觉就做完）。
-检查过程：医生将柔软的膀胱镜经尿道放入膀胱，仔细观察整个膀胱内壁是否有复发或新生的肿瘤。整个过程通常持续515分钟。
-术后观察：检查后，在观察区休息30分钟到1小时左右，若无特殊不适（如严重血尿、剧痛），即可在家人陪同下回家。
+   预约：按医生嘱咐的复查时间提前预约。
+   术前准备：检查前可能需要做简单的尿常规、感染筛查（如HIV、梅毒、乙肝等，这是常规手术前检查）。部分医院要求检查前禁食水几小时（尤其是如果需要麻醉的话）。
+   麻醉：通常采用 “尿道表面麻醉” （将局麻药凝胶挤入尿道，等待数分钟起效）。对于疼痛敏感、焦虑或尿道狭窄的患者，可以选择 “静脉镇静麻醉” （即短时间的全麻，睡一觉就做完）。
+   检查过程：医生将柔软的膀胱镜经尿道放入膀胱，仔细观察整个膀胱内壁是否有复发或新生的肿瘤。整个过程通常持续515分钟。
+   术后观察：检查后，在观察区休息30分钟到1小时左右，若无特殊不适（如严重血尿、剧痛），即可在家人陪同下回家。
 3.  优点：方便快捷，节省时间和费用，患者无需在医院过夜。
 哪些特殊情况可能需要住院或特殊处理？
 虽然大部分是门诊操作，但以下情况可能需要考虑住院或更复杂的安排：
 1.  镜下发现可疑肿瘤需要同时治疗：
-如果复查时发现明确的复发小肿瘤，医生可能会 “顺便” 在麻醉下直接进行 “经尿道膀胱肿瘤电切术” 。
-这属于一个治疗性手术，而不是单纯的检查。术后可能需要留置导尿管，并可能需要住院观察12天，特别是如果止血需要、或切除范围较大时。
+   如果复查时发现明确的复发小肿瘤，医生可能会 “顺便” 在麻醉下直接进行 “经尿道膀胱肿瘤电切术” 。
+   这属于一个治疗性手术，而不是单纯的检查。术后可能需要留置导尿管，并可能需要住院观察12天，特别是如果止血需要、或切除范围较大时。
 2.  患者基础情况复杂：
-年龄非常大、有严重心肺疾病、凝血功能障碍等麻醉高危因素的患者，为了安全起见，医生可能会建议短期住院进行检查。
+   年龄非常大、有严重心肺疾病、凝血功能障碍等麻醉高危因素的患者，为了安全起见，医生可能会建议短期住院进行检查。
 3.  出现严重并发症（罕见）：
-检查后若出现大出血、严重感染、尿道损伤或膀胱穿孔等急性并发症，则需要立即住院处理。
+   检查后若出现大出血、严重感染、尿道损伤或膀胱穿孔等急性并发症，则需要立即住院处理。
 给您的复查准备建议
 1.  明确医嘱：每次复查时，一定向医生确认下一次复查是 “单纯膀胱镜检查” 还是 “膀胱镜检查+可能电切术” ，以便做好相应准备（如请假时间、陪同安排）。
 2.  沟通麻醉方式：主动与医生沟通您对疼痛的耐受度和焦虑程度，共同决定使用表面麻醉还是静脉麻醉。
 3.  安排陪同：即使门诊检查，也必须有人陪同。因为检查后可能会有短暂头晕（麻药影响）或排尿不适，且不适合自行驾车。
 4.  检查后护理：
-检查后多喝水，促进排尿，减轻尿道刺激和预防感染。
-可能会有轻微血尿和排尿刺痛感，通常12天内会自行消失。
-如果出现发热、持续加重的血尿、无法排尿或剧烈腹痛，需立即返院就诊。
+   检查后多喝水，促进排尿，减轻尿道刺激和预防感染。
+   可能会有轻微血尿和排尿刺痛感，通常12天内会自行消失。
+   如果出现发热、持续加重的血尿、无法排尿或剧烈腹痛，需立即返院就诊。
 总结：
 请放心，对于规律的术后复查，膀胱镜是一项成熟、常规的门诊操作，目的是用最小的创伤完成最重要的监测。您只需按医嘱预约，做好门诊准备即可。如果医生判断需要住院，通常会提前告知原因（如怀疑复发需准备手术）。</t>
         </is>
@@ -6131,8 +6096,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌复查膀胱镜需要住院吗？
-男性膀胱癌患者复查膀胱镜不一定需要住院，具体取决于检查方式、患者病情及医院的诊疗流程，主要分为两种情况：
+          <t>男性膀胱癌患者复查膀胱镜不一定需要住院，具体取决于检查方式、患者病情及医院的诊疗流程，主要分为两种情况：
 一、 门诊膀胱镜检查（无需住院）
 这是绝大多数患者的常规复查方式，适用于低中危非肌层浸润性膀胱癌术后、病情稳定且无明显并发症的患者。
 适用场景
@@ -6192,8 +6156,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌复查膀胱镜需要住院吗？
-男性膀胱癌复查膀胱镜是否需要住院，主要取决于检查目的、患者身体状况及医院流程，并非绝对。
+          <t>男性膀胱癌复查膀胱镜是否需要住院，主要取决于检查目的、患者身体状况及医院流程，并非绝对。
 一、通常不需要住院的情况（门诊/日间）
 常规复查膀胱镜：
 对于病情稳定、只是进行常规复查（如观察术后创面愈合、有无复发迹象）的患者，大多数医院会安排在门诊或日间病房进行。
@@ -6245,24 +6208,23 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>deepeek_raw.docx</t>
+          <t>deepseek_raw.docx</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>20.男性膀胱癌术后家庭换尿袋方法
-为男性膀胱癌术后患者（尤其是行回肠膀胱术，即腹壁造口）的家庭更换尿袋是一项非常重要的护理技能。掌握正确的方法可以有效预防感染、保护造口周围皮肤、提高患者舒适度和生活质量。
+          <t>为男性膀胱癌术后患者（尤其是行回肠膀胱术，即腹壁造口）的家庭更换尿袋是一项非常重要的护理技能。掌握正确的方法可以有效预防感染、保护造口周围皮肤、提高患者舒适度和生活质量。
 以下为您提供一份清晰、安全的 “家庭更换尿袋（造口袋）标准操作流程” ，请务必在医护人员首次指导下进行，并熟记要点。
-核心原则：清洁、干燥、无损伤
+ 核心原则：清洁、干燥、无损伤
 一、准备工作（备齐所有物品）
 1.  环境：选择干净、明亮、温暖的房间，关闭门窗避免对流风。
 2.  物品（确保都是清洁或无菌的）：
-新的造口袋（一件式或两件式，根据患者习惯）。
-造口测量尺/剪刀（用于裁剪底盘开口）。
-皮肤保护用品：造口护肤粉、皮肤保护膜（液体或喷雾）、防漏膏/环（可选）。
-清洁用品：温水、柔软小毛巾或纱布、不含酒精的温和湿巾。
-垃圾袋（用于丢弃旧造口袋）。
-镜子（帮助患者自己操作时观看）。
+    新的造口袋（一件式或两件式，根据患者习惯）。
+    造口测量尺/剪刀（用于裁剪底盘开口）。
+    皮肤保护用品：造口护肤粉、皮肤保护膜（液体或喷雾）、防漏膏/环（可选）。
+    清洁用品：温水、柔软小毛巾或纱布、不含酒精的温和湿巾。
+    垃圾袋（用于丢弃旧造口袋）。
+    镜子（帮助患者自己操作时观看）。
 二、标准操作七步法
 第一步：洗净双手
 操作者用肥皂和流动水彻底洗手。
@@ -6275,50 +6237,50 @@
 用温水浸湿的柔软毛巾或纱布，轻轻蘸洗造口和周围皮肤。
 顺序：从造口向外周环形清洗。
 关键：
-造口黏膜（红色部分）有少量毛细血管出血是正常的，轻轻压迫即可止血。
-切勿使用任何刺激性物品：如酒精、碘伏、肥皂、沐浴露等，它们会损伤皮肤和黏膜。
-清洗后用干纱布或软布轻轻拍干皮肤，保持完全干燥。潮湿是导致皮肤问题和粘贴不牢的主要原因。
+    造口黏膜（红色部分）有少量毛细血管出血是正常的，轻轻压迫即可止血。
+    切勿使用任何刺激性物品：如酒精、碘伏、肥皂、沐浴露等，它们会损伤皮肤和黏膜。
+    清洗后用干纱布或软布轻轻拍干皮肤，保持完全干燥。潮湿是导致皮肤问题和粘贴不牢的主要原因。
 第四步：观察与评估（非常重要！）
 观察造口：颜色应为鲜红或粉红色，湿润。如变为暗红、紫黑或苍白，需联系医生。
 观察周围皮肤：有无发红、破损、皮疹、溃疡或瘙痒。根据情况处理：
-正常皮肤：可直接进入下一步。
-轻微发红/潮湿：喷洒造口护肤粉，停留30秒后轻轻扫去多余粉末，再喷皮肤保护膜形成隔离层。
-皮肤有凹陷或不平：使用防漏膏或防漏环填补，使其平整。
+    正常皮肤：可直接进入下一步。
+    轻微发红/潮湿：喷洒造口护肤粉，停留30秒后轻轻扫去多余粉末，再喷皮肤保护膜形成隔离层。
+    皮肤有凹陷或不平：使用防漏膏或防漏环填补，使其平整。
 第五步：测量与裁剪
 用测量尺准确测量造口根部的直径。
 在新造口袋的底盘背面，根据测量结果裁剪开口。
-开口大小是关键：应比造口根部大12毫米。过大会导致皮肤暴露，受尿液侵蚀；过小会摩擦挤压造口黏膜，导致出血或水肿。
+    开口大小是关键：应比造口根部大12毫米。过大会导致皮肤暴露，受尿液侵蚀；过小会摩擦挤压造口黏膜，导致出血或水肿。
 第六步：粘贴新造口袋
 1.  预热底盘：用手心捂住底盘背面的医用黏胶几分钟，使其软化，粘贴效果更好。
 2.  对准粘贴：
-请患者坐直或躺平，使腹部皮肤无褶皱。
-撕去底盘背面的保护纸。
-从下往上对准造口，确保造口从裁剪的孔中完全露出。
-先粘贴底盘下部，然后由下至上、由内向外轻轻抚平底盘，排出空气，确保粘贴紧密无褶皱。
+    请患者坐直或躺平，使腹部皮肤无褶皱。
+    撕去底盘背面的保护纸。
+    从下往上对准造口，确保造口从裁剪的孔中完全露出。
+    先粘贴底盘下部，然后由下至上、由内向外轻轻抚平底盘，排出空气，确保粘贴紧密无褶皱。
 3.  按压加固：用手掌以画圈方式按压底盘510分钟，利用体温使黏胶与皮肤更好融合。
 第七步：连接与检查
 如果使用两件式造口袋，将袋子扣在底盘上，听到“咔哒”声表示已锁紧。
 确保造口袋的引流阀处于关闭状态。
 最后，用手再次检查底盘边缘是否贴合紧密。
-三、关键注意事项与问题处理
+ 三、关键注意事项与问题处理
 1.  更换频率：
-底盘：一般37天更换一次，出现渗漏、卷边、皮肤瘙痒或异味时立即更换。避免频繁更换损伤皮肤。
-尿袋：每天清洗（用清水即可），建议12个月更换新袋。
+    底盘：一般37天更换一次，出现渗漏、卷边、皮肤瘙痒或异味时立即更换。避免频繁更换损伤皮肤。
+    尿袋：每天清洗（用清水即可），建议12个月更换新袋。
 2.  渗漏处理：
-一旦发现渗漏，必须立即更换，不要尝试修补。
-分析原因：是否裁剪过大？皮肤不平未使用防漏膏？粘贴时腹部有褶皱？
+    一旦发现渗漏，必须立即更换，不要尝试修补。
+    分析原因：是否裁剪过大？皮肤不平未使用防漏膏？粘贴时腹部有褶皱？
 3.  尿液处理与清洁：
-尿袋不要超过2/3满就要排放，防止过重导致底盘脱落。
-排放尿液后，用清水冲洗尿袋末端，保持清洁。
-晚上可连接大容量夜用尿袋，保证睡眠。
+    尿袋不要超过2/3满就要排放，防止过重导致底盘脱落。
+    排放尿液后，用清水冲洗尿袋末端，保持清洁。
+    晚上可连接大容量夜用尿袋，保证睡眠。
 4.  活动与着装：
-可正常沐浴（粘贴底盘淋浴，或取下底盘淋浴后迅速擦干皮肤再粘贴）。沐浴时可在底盘周围贴一圈防水胶带。
-穿着宽松柔软的内裤和裤子，避免腰带直接压迫造口。
+    可正常沐浴（粘贴底盘淋浴，或取下底盘淋浴后迅速擦干皮肤再粘贴）。沐浴时可在底盘周围贴一圈防水胶带。
+    穿着宽松柔软的内裤和裤子，避免腰带直接压迫造口。
 5.  何时就医：
-造口颜色变暗、发黑、严重回缩或突出。
-周围皮肤严重溃烂、疼痛无法缓解。
-出现发热、腹痛、尿液浑浊恶臭（可能感染）。
-四、心理支持
+    造口颜色变暗、发黑、严重回缩或突出。
+    周围皮肤严重溃烂、疼痛无法缓解。
+    出现发热、腹痛、尿液浑浊恶臭（可能感染）。
+ 四、心理支持
 操作者动作要自信、轻柔，多鼓励患者。
 鼓励患者逐步学习自己更换，重获自理能力，对建立信心非常重要。
 最后建议：在患者出院前，务必请求医院的造口治疗师（ET）或专科护士进行手把手教学和考核，他们是您最好的老师。也可以购买一些造口护理模型在家练习。
@@ -6359,8 +6321,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌术后家庭换尿袋方法
-男性膀胱癌术后（尤其是尿流改道术后，如回肠膀胱、输尿管皮肤造口），家庭换尿袋是一项需要规范操作的护理技能，核心原则是 无菌操作、轻柔固定、防漏防感染，具体步骤和注意事项如下：
+          <t>男性膀胱癌术后（尤其是尿流改道术后，如回肠膀胱、输尿管皮肤造口），家庭换尿袋是一项需要规范操作的护理技能，核心原则是 无菌操作、轻柔固定、防漏防感染，具体步骤和注意事项如下：
 一、 准备用物
 核心物品
 一次性造口袋（根据造口类型选择：一件式 / 两件式，建议选防漏、透气款）；
@@ -6437,49 +6398,49 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>男性膀胱癌术后家庭换尿袋方法
-男性膀胱癌术后家庭更换尿袋（通常指尿路造口袋）是一项重要的护理技能，掌握正确的方法可以减少感染风险、提高舒适度并保持皮肤健康。以下是详细的步骤和注意事项：
+          <t>男性膀胱癌术后家庭更换尿袋（通常指尿路造口袋）是一项重要的护理技能，掌握正确的方法可以减少感染风险、提高舒适度并保持皮肤健康。以下是详细的步骤和注意事项：
 一、准备工作
 1.  物品准备：
-◦   新的尿路造口袋（底盘和袋子）。
-◦   温水、柔软的毛巾或纱布。
-◦   医用剪刀（如需裁剪底盘）。
-◦   温和的皮肤清洁剂（如无酒精湿巾）。
-◦   干燥的皮肤保护粉或皮肤屏障膜（可选，用于保护周围皮肤）。
-◦   垃圾袋。
-◦   手套（可选，保持卫生）。
+    ◦   新的尿路造口袋（底盘和袋子）。
+    ◦   温水、柔软的毛巾或纱布。
+    ◦   医用剪刀（如需裁剪底盘）。
+    ◦   温和的皮肤清洁剂（如无酒精湿巾）。
+    ◦   干燥的皮肤保护粉或皮肤屏障膜（可选，用于保护周围皮肤）。
+    ◦   垃圾袋。
+    ◦   手套（可选，保持卫生）。
 2.  环境准备：
-◦   选择一个光线充足、温暖、私密且干净的空间。
-◦   在操作台上铺上干净的毛巾或纸巾。
+    ◦   选择一个光线充足、温暖、私密且干净的空间。
+    ◦   在操作台上铺上干净的毛巾或纸巾。
 3.  个人准备：
-◦   操作者洗净双手，最好戴上干净的手套。
-◦   让患者采取舒适的体位，如平卧位或半卧位，充分暴露造口部位。
+    ◦   操作者洗净双手，最好戴上干净的手套。
+    ◦   让患者采取舒适的体位，如平卧位或半卧位，充分暴露造口部位。
 二、更换步骤
 1.  取下旧造口袋：
-◦   一手轻轻按压造口周围的皮肤，另一手慢慢将旧造口袋从皮肤上揭下。动作要轻柔，避免用力撕扯损伤皮肤。
-◦   如果底盘粘贴较紧，可以用温水浸湿底盘边缘，使其更容易剥离。
+    ◦   一手轻轻按压造口周围的皮肤，另一手慢慢将旧造口袋从皮肤上揭下。动作要轻柔，避免用力撕扯损伤皮肤。
+    ◦   如果底盘粘贴较紧，可以用温水浸湿底盘边缘，使其更容易剥离。
 2.  清洁造口及周围皮肤：
-◦   用温水或温和的皮肤清洁剂清洗造口及周围皮肤。
-◦   用柔软的毛巾或纱布轻轻拍干，或用吹风机冷风档吹干。确保皮肤干燥，无残留水分或清洁剂。
-◦   检查造口是否有红肿、破损、出血、分泌物异常等情况，并记录。
+    ◦   用温水或温和的皮肤清洁剂清洗造口及周围皮肤。
+    ◦   用柔软的毛巾或纱布轻轻拍干，或用吹风机冷风档吹干。确保皮肤干燥，无残留水分或清洁剂。
+    ◦   检查造口是否有红肿、破损、出血、分泌物异常等情况，并记录。
 3.  测量造口大小（如需要）：
-◦   使用造口尺测量造口的直径。
-◦   根据测量结果，用剪刀修剪新底盘的中心孔。中心孔应比造口实际直径大1-2毫米，以确保造口能轻松伸入而不压迫周围组织。
-◦   修剪时注意底盘边缘光滑，无毛刺。
+    ◦   使用造口尺测量造口的直径。
+    ◦   根据测量结果，用剪刀修剪新底盘的中心孔。中心孔应比造口实际直径大1-2毫米，以确保造口能轻松伸入而不压迫周围组织。
+    ◦   修剪时注意底盘边缘光滑，无毛刺。
 4.  粘贴新底盘：
-◦   撕去新底盘背面的保护纸。
-◦   将底盘中心孔对准造口，轻轻贴上。用手指由内向外、由中心向四周均匀按压底盘，确保其平整、牢固地粘贴在皮肤上。特别注意底盘的边缘部分要压实。
-◦   如果是两件式造口袋，粘贴好底盘后，再将袋子与底盘连接好。
+    ◦   撕去新底盘背面的保护纸。
+    ◦   将底盘中心孔对准造口，轻轻贴上。用手指由内向外、由中心向四周均匀按压底盘，确保其平整、牢固地粘贴在皮肤上。特别注意底盘的边缘部分要压实。
+    ◦   如果是两件式造口袋，粘贴好底盘后，再将袋子与底盘连接好。
 5.  整理与固定：
-◦   确保造口袋妥善固定在衣物下方，避免牵拉或扭曲。
-◦   检查连接处是否紧密，防止尿液渗漏。
-◦   妥善处理旧造口袋和废弃物。</t>
+    ◦   确保造口袋妥善固定在衣物下方，避免牵拉或扭曲。
+    ◦   检查连接处是否紧密，防止尿液渗漏。
+    ◦   妥善处理旧造口袋和废弃物。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -14273,7 +14234,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025 edition; official archive</t>
+          <t>2024 guideline update (EAU NMIBC guideline update); cited 2024 publication</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>